<commit_message>
Workbook: C15 cap wording matches prototype; no standard for retirement/plan-until age
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhUEAkgdki1q9EpFqaquGU
</commit_message>
<xml_diff>
--- a/deliverables/LifeGoals-Calculators.xlsx
+++ b/deliverables/LifeGoals-Calculators.xlsx
@@ -1416,7 +1416,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Generally the standard is 66, when the State Pension is paid (you can usually draw a pension from 60, some schemes from 50). Choose what you want to use. Example only: 65.</t>
+          <t xml:space="preserve">You can usually draw a pension from 60 (some schemes from 50); State Pension is paid from 66. Choose your own: there is no default. Example only: 65.</t>
         </r>
       </text>
     </comment>
@@ -1962,7 +1962,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Generally the standard is 66, when the State Pension is paid (you can usually draw a pension from 60, some schemes from 50). Choose what you want to use. Example only: 66.</t>
+          <t xml:space="preserve">You can usually draw a pension from 60 (some schemes from 50); State Pension is paid from 66. Choose your own: there is no default. Example only: 66.</t>
         </r>
       </text>
     </comment>
@@ -1974,7 +1974,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Generally the standard is to plan to 90–95: at 65, average life expectancy in Ireland is about 83 for men and 86 for women (CSO). Choose what you want to use. Example only: 90.</t>
+          <t xml:space="preserve">At 65, average life expectancy in Ireland is about 83 for men and 86 for women (CSO); many people plan to 90–95. Choose your own: there is no default. Example only: 90.</t>
         </r>
       </text>
     </comment>
@@ -4290,7 +4290,7 @@
     <t xml:space="preserve">• Open a calculator from the list below. Fill the yellow cells (blue text): everything else updates on its own.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Every number is one of three types (journey spec §14). Type 1, set by Government (tax, USC, PRSI, relief %, lump-sum bands, DIRT, exit tax, Central Bank limits, full State Pension and benefit rates): on the Assumptions sheet, not an input. Type 2, varies within a known range (mortgage rate, card APR, fund charges, the State Pension you will get …): a yellow input with "Usually between X and Y (source)". Type 3, personal (inflation, growth, pay rises, emergency months, drawdown timing, retirement multiple, retirement age, plan-until age, and your own figures): a yellow input left BLANK with "Generally the standard is X (source). Choose what you want to use."</t>
+    <t xml:space="preserve">• Every number is one of three types (journey spec §14). Type 1, set by Government (tax, USC, PRSI, relief %, lump-sum bands, DIRT, exit tax, Central Bank limits, full State Pension and benefit rates): on the Assumptions sheet, not an input. Type 2, varies within a known range (mortgage rate, card APR, fund charges, the State Pension you will get …): a yellow input with "Usually between X and Y (source)". Type 3, personal (inflation, growth, pay rises, emergency months, drawdown timing, retirement multiple, and your own figures): a yellow input left BLANK with "Generally the standard is X (source). Choose what you want to use." Retirement age and plan-until age are blank with guidance only, never a standard.</t>
   </si>
   <si>
     <t xml:space="preserve">• Blank inputs stay blank: results that need them show "Choose your … to see this". Switch "Fill example values?" (above) to Yes to fill every blank input with its grey "Example only" figure (the standard, or the sample customer's figure).</t>
@@ -4818,7 +4818,7 @@
     <t xml:space="preserve">UI/UX Appendix B</t>
   </si>
   <si>
-    <t xml:space="preserve">Singular "1 month"; C15 at the 60-year cap reads "Lasts 60+ years: beyond your plan age" (not "age 126"); C13/C14 show the relief room left after what you already pay in.</t>
+    <t xml:space="preserve">Singular "1 month"; C15 at the 60-year cap reads "Beyond [plan-until age] (your plan-until age)", as the prototype (not "age 126"); C13/C14 show the relief room left after what you already pay in.</t>
   </si>
   <si>
     <t xml:space="preserve">Remove the placeholder "[confirm current Central Bank rules]" from the customer line (prototype copy; the workbook uses the audit's replacement wording).</t>
@@ -6429,7 +6429,7 @@
     <t xml:space="preserve">Target retirement age</t>
   </si>
   <si>
-    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 66, when the State Pension is paid (you can usually draw a pension from 60, some schemes from 50). Choose what you want to use. Allowed: 50 to 75 · steps of 1</t>
+    <t xml:space="preserve">Type 3 · your choice (no standard) · You can usually draw a pension from 60 (some schemes from 50); State Pension is paid from 66. Choose your own: there is no default. Allowed: 50 to 75 · steps of 1</t>
   </si>
   <si>
     <t xml:space="preserve">Pension value today</t>
@@ -6930,13 +6930,13 @@
     <t xml:space="preserve">Your age when withdrawals start</t>
   </si>
   <si>
-    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 66, when the State Pension is paid (you can usually draw a pension from 60, some schemes from 50). Choose what you want to use. Allowed: 50 to 90 · steps of 1</t>
+    <t xml:space="preserve">Type 3 · your choice (no standard) · You can usually draw a pension from 60 (some schemes from 50); State Pension is paid from 66. Choose your own: there is no default. Allowed: 50 to 90 · steps of 1</t>
   </si>
   <si>
     <t xml:space="preserve">Plan to age</t>
   </si>
   <si>
-    <t xml:space="preserve">Type 3 · your choice · Generally the standard is to plan to 90–95: at 65, average life expectancy in Ireland is about 83 for men and 86 for women (CSO). Choose what you want to use. Allowed: 85 to 100 · steps of 1</t>
+    <t xml:space="preserve">Type 3 · your choice (no standard) · At 65, average life expectancy in Ireland is about 83 for men and 86 for women (CSO); many people plan to 90–95. Choose your own: there is no default. Allowed: 85 to 100 · steps of 1</t>
   </si>
   <si>
     <t xml:space="preserve">ƒx  =IF(NOT(ISBLANK(Stmt_Projected_Fund)),Stmt_Projected_Fund,IF(NOT(ISBLANK(Stmt_Fund_Value)),Stmt_Fund_Value,Retirement_Savings))</t>
@@ -6951,7 +6951,7 @@
     <t xml:space="preserve">Money lasts to about age</t>
   </si>
   <si>
-    <t xml:space="preserve">ƒx  =IF(ISNUMBER(Years_Lasting),IF(Years_Lasting&gt;=Cap_Years,Cap_Years&amp;"+ years",Age_At_Start+Years_Lasting),"Choose your inflation rate to see this")</t>
+    <t xml:space="preserve">ƒx  =IF(ISNUMBER(Years_Lasting),IF(Years_Lasting&gt;=Cap_Years,"Beyond "&amp;Plan_To_Age&amp;" (your plan-until age)",Age_At_Start+Years_Lasting),"Choose your inflation rate to see this")</t>
   </si>
   <si>
     <t xml:space="preserve">Withdrawal rate (first year)</t>
@@ -11841,7 +11841,7 @@
       </c>
       <c r="E114" s="18"/>
     </row>
-    <row r="115" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B115" s="11" t="s">
         <v>181</v>
       </c>
@@ -13342,13 +13342,13 @@
       <formula1>1</formula1>
       <formula2>40</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 0% to 5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: %. Allowed: 0% to 5%." promptTitle="Annual charges % (if shown)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C12" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0.05</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €100,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €100,000,000." promptTitle="Total value" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C11" type="decimal">
       <formula1>0</formula1>
       <formula2>100000000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: %. Allowed: 0% to 5%." promptTitle="Annual charges % (if shown)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C12" type="decimal">
-      <formula1>0</formula1>
-      <formula2>0.05</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €500 to €5,000,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure. In the app it is pre-filled from Your finances / statement: investments.  Allowed: €500 to €5,000,000 · steps of €100." promptTitle="Amount" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C16" type="decimal">
       <formula1>500</formula1>
@@ -14818,14 +14818,6 @@
       <formula1>0</formula1>
       <formula2>0.1</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: %. Allowed: 0% to 5%." promptTitle="Annual charges % (if shown)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="decimal">
-      <formula1>0</formula1>
-      <formula2>0.05</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 2.5% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between 0.5% and 1.5% a year for pension charges (your statement shows yours). Enter your own figure.  Allowed: 0% to 2.5% · steps of 0.05%." promptTitle="Typical pension charges (if your" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C30" type="decimal">
-      <formula1>0</formula1>
-      <formula2>0.025</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €50,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €50,000,000." promptTitle="Fund value today" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C11" type="decimal">
       <formula1>0</formula1>
       <formula2>50000000</formula2>
@@ -14850,11 +14842,15 @@
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 0% to 5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: %. Allowed: 0% to 5%." promptTitle="Annual charges % (if shown)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0.05</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter 20 to 70 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure. In the app it is pre-filled from About you: age.  Allowed: 20 to 70 · steps of 1." promptTitle="Your age" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C21" type="whole">
       <formula1>20</formula1>
       <formula2>70</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 50 to 75 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 66, when the State Pension is paid (you can usually draw a pension from 60, some schemes from 50). Choose what you want to use.  Allowed: 50 to 75 · steps of 1." promptTitle="Target retirement age" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C22" type="whole">
+    <dataValidation allowBlank="true" error="Please enter 50 to 75 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="You can usually draw a pension from 60 (some schemes from 50); State Pension is paid from 66. Choose your own: there is no default.  Allowed: 50 to 75 · steps of 1." promptTitle="Target retirement age" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C22" type="whole">
       <formula1>50</formula1>
       <formula2>75</formula2>
     </dataValidation>
@@ -14885,6 +14881,10 @@
     <dataValidation allowBlank="true" error="Please enter 20 to 33 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 25 times the yearly income you need (about 4% a year). Choose what you want to use.  Allowed: 20 to 33 · steps of 1." promptTitle="Retirement savings target: × the" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C29" type="whole">
       <formula1>20</formula1>
       <formula2>33</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 0% to 2.5% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between 0.5% and 1.5% a year for pension charges (your statement shows yours). Enter your own figure.  Allowed: 0% to 2.5% · steps of 0.05%." promptTitle="Typical pension charges (if your" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C30" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0.025</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter 0% to 25% · steps of 1%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 25% of the fund, the most allowed (first €200,000 tax-free, next €300,000 at 20%). Choose what you want to use.  Allowed: 0% to 25% · steps of 1%." promptTitle="Tax-free lump sum you plan to ta" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C31" type="decimal">
       <formula1>0</formula1>
@@ -15568,6 +15568,10 @@
       <formula1>0</formula1>
       <formula2>0.05</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 0% to 2.5% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between 0.5% and 1.5% a year for pension charges (your statement shows yours). Enter your own figure.  Allowed: 0% to 2.5% · steps of 0.05%." promptTitle="Typical pension charges (if your" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C19" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0.025</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €15,000 to €2,500,000 · steps of €1,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure. In the app it is pre-filled from Your finances: income.  Allowed: €15,000 to €2,500,000 · steps of €1,000." promptTitle="Salary" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C15" type="decimal">
       <formula1>15000</formula1>
       <formula2>2500000</formula2>
@@ -15583,10 +15587,6 @@
     <dataValidation allowBlank="true" error="Please enter 1% to 7% · steps of 0.5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use.  Allowed: 1% to 7% · steps of 0.5%." promptTitle="Growth assumption a year" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
       <formula1>0.01</formula1>
       <formula2>0.07</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 2.5% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between 0.5% and 1.5% a year for pension charges (your statement shows yours). Enter your own figure.  Allowed: 0% to 2.5% · steps of 0.05%." promptTitle="Typical pension charges (if your" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C19" type="decimal">
-      <formula1>0</formula1>
-      <formula2>0.025</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter 20% or 40%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between 20% or 40%: your top rate of income tax (the Tax engine works it out). In the app it is pre-filled from Tax engine marginal rate (band by status: €44k single, €48k single parent, €53k married, + up to €35k second earne Allowed: 20% or 40%." promptTitle="Your tax rate (0.2 = 20%, 0.4 = " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C20" type="list">
       <formula1>"0.2,0.4"</formula1>
@@ -16281,13 +16281,13 @@
       <formula1>0</formula1>
       <formula2>0.05</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 0% to 2.5% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between 0.5% and 1.5% a year for pension charges (your statement shows yours). Enter your own figure.  Allowed: 0% to 2.5% · steps of 0.05%." promptTitle="Typical pension charges (if your" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C19" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0.025</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter 1% to 7% · steps of 0.5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use.  Allowed: 1% to 7% · steps of 0.5%." promptTitle="Growth assumption a year" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
       <formula1>0.01</formula1>
       <formula2>0.07</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 2.5% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between 0.5% and 1.5% a year for pension charges (your statement shows yours). Enter your own figure.  Allowed: 0% to 2.5% · steps of 0.05%." promptTitle="Typical pension charges (if your" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C19" type="decimal">
-      <formula1>0</formula1>
-      <formula2>0.025</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter 18 to 75 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure. In the app it is pre-filled from About you: age.  Allowed: 18 to 75 · steps of 1." promptTitle="Your age (for the pension relief" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C21" type="whole">
       <formula1>18</formula1>
@@ -16674,11 +16674,11 @@
         <v>893</v>
       </c>
       <c r="C29" s="61" t="str">
-        <f aca="false">IF(Need_2&lt;&gt;"",Need_2,IF(ISNUMBER(Years_Lasting),IF(Years_Lasting&gt;=Cap_Years,Cap_Years&amp;"+ years",Age_At_Start+Years_Lasting),"Choose your inflation rate to see this"))</f>
+        <f aca="false">IF(Need_2&lt;&gt;"",Need_2,IF(ISNUMBER(Years_Lasting),IF(Years_Lasting&gt;=Cap_Years,"Beyond "&amp;Plan_To_Age&amp;" (your plan-until age)",Age_At_Start+Years_Lasting),"Choose your inflation rate to see this"))</f>
         <v>Choose your inflation rate to see this</v>
       </c>
       <c r="D29" s="62" t="str">
-        <f aca="false">IF(Need_2&lt;&gt;"",Need_2,IF(ISNUMBER(Years_Lasting),IF(Years_Lasting&gt;=Cap_Years,"Lasts "&amp;Cap_Years&amp;"+ years: beyond your plan age ("&amp;Plan_To_Age&amp;")",IF(Age_At_Start+Years_Lasting&gt;=Plan_To_Age,"Lasts to your plan age ("&amp;Plan_To_Age&amp;")","Runs out "&amp;(Plan_To_Age-Age_At_Start-Years_Lasting)&amp;" years before your plan age")),"Choose your inflation rate to see this"))</f>
+        <f aca="false">IF(Need_2&lt;&gt;"",Need_2,IF(ISNUMBER(Years_Lasting),IF(Years_Lasting&gt;=Cap_Years,"Beyond "&amp;Plan_To_Age&amp;" (your plan-until age)",IF(Age_At_Start+Years_Lasting&gt;=Plan_To_Age,"Lasts to your plan age ("&amp;Plan_To_Age&amp;")","Runs out "&amp;(Plan_To_Age-Age_At_Start-Years_Lasting)&amp;" years before your plan age")),"Choose your inflation rate to see this"))</f>
         <v>Choose your inflation rate to see this</v>
       </c>
       <c r="E29" s="41" t="s">
@@ -18148,11 +18148,11 @@
       <formula1>"Start of year,End of year"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 50 to 90 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 66, when the State Pension is paid (you can usually draw a pension from 60, some schemes from 50). Choose what you want to use.  Allowed: 50 to 90 · steps of 1." promptTitle="Your age when withdrawals start" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C20" type="whole">
+    <dataValidation allowBlank="true" error="Please enter 50 to 90 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="You can usually draw a pension from 60 (some schemes from 50); State Pension is paid from 66. Choose your own: there is no default.  Allowed: 50 to 90 · steps of 1." promptTitle="Your age when withdrawals start" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C20" type="whole">
       <formula1>50</formula1>
       <formula2>90</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 85 to 100 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is to plan to 90–95: at 65, average life expectancy in Ireland is about 83 for men and 86 for women (CSO). Choose what you want to use.  Allowed: 85 to 100 · steps of 1." promptTitle="Plan to age" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C21" type="whole">
+    <dataValidation allowBlank="true" error="Please enter 85 to 100 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="At 65, average life expectancy in Ireland is about 83 for men and 86 for women (CSO); many people plan to 90–95. Choose your own: there is no default.  Allowed: 85 to 100 · steps of 1." promptTitle="Plan to age" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C21" type="whole">
       <formula1>85</formula1>
       <formula2>100</formula2>
     </dataValidation>
@@ -22545,10 +22545,6 @@
     <mergeCell ref="B40:E40"/>
   </mergeCells>
   <dataValidations count="9">
-    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C13" type="whole">
-      <formula1>1</formula1>
-      <formula2>30</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €15,000 to €2,500,000 · steps of €1,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure. In the app it is pre-filled from Your finances: income.  Allowed: €15,000 to €2,500,000 · steps of €1,000." promptTitle="Your gross yearly income" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C6" type="decimal">
       <formula1>15000</formula1>
       <formula2>2500000</formula2>
@@ -22576,6 +22572,10 @@
     <dataValidation allowBlank="true" error="Please enter €0 to €10,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between €2,500 and €3,500 for legal and survey fees (stamp duty is added for you). Enter your own figure.  Allowed: €0 to €10,000 · steps of €100." promptTitle="Legal and other buying fees" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C12" type="decimal">
       <formula1>0</formula1>
       <formula2>10000</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C13" type="whole">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €500,000 · steps of €1,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Optional: leave blank for none.  Allowed: €0 to €500,000 · steps of €1,000." promptTitle="What if: save extra towards the " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C14" type="decimal">
       <formula1>0</formula1>
@@ -23068,13 +23068,13 @@
       <formula1>1</formula1>
       <formula2>40</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 0% to 5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: %. Allowed: 0% to 5%." promptTitle="Annual charges % (if shown)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C8" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0.05</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €100,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €100,000,000." promptTitle="Total value" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="decimal">
       <formula1>0</formula1>
       <formula2>100000000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: %. Allowed: 0% to 5%." promptTitle="Annual charges % (if shown)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C8" type="decimal">
-      <formula1>0</formula1>
-      <formula2>0.05</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter 0% to 8% · steps of 0.5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 5% a year before charges and tax for a mixed fund (long-run 5%–6% a year; Irish rules audit B3). Choose what you want to use.  Allowed: 0% to 8% · steps of 0.5%." promptTitle="Growth a year (before fees)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C14" type="decimal">
       <formula1>0</formula1>
@@ -25944,13 +25944,13 @@
       <formula1>0</formula1>
       <formula2>10000000</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter €0 to €50,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €50,000,000." promptTitle="Fund value today" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9" type="decimal">
+      <formula1>0</formula1>
+      <formula2>50000000</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €100,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €100,000,000." promptTitle="Total value" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C10" type="decimal">
       <formula1>0</formula1>
       <formula2>100000000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter €0 to €50,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €50,000,000." promptTitle="Fund value today" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9" type="decimal">
-      <formula1>0</formula1>
-      <formula2>50000000</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €100,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €100,000,000." promptTitle="Property value (valuation)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C8" type="decimal">
       <formula1>0</formula1>
@@ -28117,6 +28117,10 @@
     <mergeCell ref="B54:E54"/>
   </mergeCells>
   <dataValidations count="11">
+    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="whole">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €10,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €10,000,000." promptTitle="Outstanding balance" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="decimal">
       <formula1>0</formula1>
       <formula2>10000000</formula2>
@@ -28152,10 +28156,6 @@
     <dataValidation allowBlank="true" error="Please enter €0 to €100,000 · steps of €1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Optional: leave blank for none.  Allowed: €0 to €100,000 · steps of €1." promptTitle="Your actual monthly repayment (o" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="decimal">
       <formula1>0</formula1>
       <formula2>100000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="whole">
-      <formula1>1</formula1>
-      <formula2>30</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter -2% to 3% · steps of 0.25%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Optional: leave blank for none.  Allowed: -2% to 3% · steps of 0.25%." promptTitle="What if: rates change by" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C19" type="decimal">
       <formula1>-0.02</formula1>
@@ -35585,13 +35585,13 @@
     <mergeCell ref="B38:E38"/>
   </mergeCells>
   <dataValidations count="12">
+    <dataValidation allowBlank="true" error="Please enter €0 to €10,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between €2,500 and €3,500 for legal and survey fees (stamp duty is added for you). Enter your own figure.  Allowed: €0 to €10,000 · steps of €100." promptTitle="Legal and other buying fees" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C15" type="decimal">
+      <formula1>0</formula1>
+      <formula2>10000</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="whole">
       <formula1>1</formula1>
       <formula2>30</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter €0 to €10,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between €2,500 and €3,500 for legal and survey fees (stamp duty is added for you). Enter your own figure.  Allowed: €0 to €10,000 · steps of €100." promptTitle="Legal and other buying fees" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C15" type="decimal">
-      <formula1>0</formula1>
-      <formula2>10000</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €100,000 to €10,000,000 · steps of €5,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €100,000 to €10,000,000 · steps of €5,000." promptTitle="Home price" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="decimal">
       <formula1>100000</formula1>

</xml_diff>

<commit_message>
Spec §15: 'Not sure? See an example' card replaces 'Estimate for me' and 'I don't have this'
Workbook document-reader precedence note updated to match (no estimates).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhUEAkgdki1q9EpFqaquGU
</commit_message>
<xml_diff>
--- a/deliverables/LifeGoals-Calculators.xlsx
+++ b/deliverables/LifeGoals-Calculators.xlsx
@@ -8355,7 +8355,7 @@
     <t xml:space="preserve">Document reader spec (for the developer building extraction)</t>
   </si>
   <si>
-    <t xml:space="preserve">• Precedence: statement figure &gt; typed figure &gt; estimate (as in the prototype: S.src doc &gt; typed &gt; est). The calculators show this in their FIGURE USED box.</t>
+    <t xml:space="preserve">• Precedence: statement figure &gt; typed figure (as in the prototype: S.src doc &gt; typed). A figure the customer has not given is Missing; nothing is estimated for them. The calculators show this in their FIGURE USED box.</t>
   </si>
   <si>
     <t xml:space="preserve">• Confidence: each extracted field carries a confidence. Below 80% (Assumptions › Reader_Confidence_Min) ask the customer to confirm the figure before it is used.</t>
@@ -22549,6 +22549,14 @@
     <mergeCell ref="B40:E40"/>
   </mergeCells>
   <dataValidations count="9">
+    <dataValidation allowBlank="true" error="Please enter €0 to €10,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between €2,500 and €3,500 for legal and survey fees (stamp duty is added for you). Enter your own figure.  Allowed: €0 to €10,000 · steps of €100." promptTitle="Legal and other buying fees" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C12" type="decimal">
+      <formula1>0</formula1>
+      <formula2>10000</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C13" type="whole">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €15,000 to €2,500,000 · steps of €1,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure. In the app it is pre-filled from Your finances: income.  Allowed: €15,000 to €2,500,000 · steps of €1,000." promptTitle="Your gross yearly income" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C6" type="decimal">
       <formula1>15000</formula1>
       <formula2>2500000</formula2>
@@ -22572,14 +22580,6 @@
     <dataValidation allowBlank="true" error="Please enter 10 to 35 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 10 to 35 · steps of 1." promptTitle="Mortgage term" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C11" type="whole">
       <formula1>10</formula1>
       <formula2>35</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter €0 to €10,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between €2,500 and €3,500 for legal and survey fees (stamp duty is added for you). Enter your own figure.  Allowed: €0 to €10,000 · steps of €100." promptTitle="Legal and other buying fees" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C12" type="decimal">
-      <formula1>0</formula1>
-      <formula2>10000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C13" type="whole">
-      <formula1>1</formula1>
-      <formula2>30</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €500,000 · steps of €1,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Optional: leave blank for none.  Allowed: €0 to €500,000 · steps of €1,000." promptTitle="What if: save extra towards the " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C14" type="decimal">
       <formula1>0</formula1>
@@ -35593,13 +35593,13 @@
       <formula1>0</formula1>
       <formula2>10000</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter €100,000 to €10,000,000 · steps of €5,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €100,000 to €10,000,000 · steps of €5,000." promptTitle="Home price" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="decimal">
+      <formula1>100000</formula1>
+      <formula2>10000000</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="whole">
       <formula1>1</formula1>
       <formula2>30</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter €100,000 to €10,000,000 · steps of €5,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €100,000 to €10,000,000 · steps of €5,000." promptTitle="Home price" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="decimal">
-      <formula1>100000</formula1>
-      <formula2>10000000</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €500 to €50,000 · steps of €50." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €500 to €50,000 · steps of €50." promptTitle="Monthly rent" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C6" type="decimal">
       <formula1>500</formula1>

</xml_diff>

<commit_message>
UI/UX spec for §15 and §16; LifeMap name in the workbook
- Spec: new section 4 (Not sure? See an example: link, card layout, dialog
  behaviour, all 33 card texts, statuses, precedence document > typed >
  Missing, worked-out figures, checklists, gaps in calculators) and section 5
  (LifeMap name, new cover, D1 title, Emergency fund tile and goal, Q8 road
  wording); gate, tags, pre-fill and Appendix A/B updated. 293 pages.
- Check: 7,155 pass, 0 fail; planted test 9/9 caught (41 fails), incl. an
  example-card sentence and the cover headline.
- Workbook: customer-facing "LifeGoals" text renamed to "LifeMap" (titles,
  labels, prompts, notes); file names, defined names and formulas unchanged.
  recalc.py: 0 errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhUEAkgdki1q9EpFqaquGU
</commit_message>
<xml_diff>
--- a/deliverables/LifeGoals-Calculators.xlsx
+++ b/deliverables/LifeGoals-Calculators.xlsx
@@ -1476,7 +1476,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use. Example only: 4.5%.</t>
+          <t xml:space="preserve">Generally the standard is 4.5% a year after charges while you work (LifeMap Standard set; Cautious 4%). Choose what you want to use. Example only: 4.5%.</t>
         </r>
       </text>
     </comment>
@@ -1488,7 +1488,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Generally the standard is 3% a year (Irish pay has grown about 3%–4% a year recently; LifeGoals Standard set). Choose what you want to use. Example only: 3%.</t>
+          <t xml:space="preserve">Generally the standard is 3% a year (Irish pay has grown about 3%–4% a year recently; LifeMap Standard set). Choose what you want to use. Example only: 3%.</t>
         </r>
       </text>
     </comment>
@@ -1654,7 +1654,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use. Example only: 4.5%.</t>
+          <t xml:space="preserve">Generally the standard is 4.5% a year after charges while you work (LifeMap Standard set; Cautious 4%). Choose what you want to use. Example only: 4.5%.</t>
         </r>
       </text>
     </comment>
@@ -1796,7 +1796,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use. Example only: 4.5%.</t>
+          <t xml:space="preserve">Generally the standard is 4.5% a year after charges while you work (LifeMap Standard set; Cautious 4%). Choose what you want to use. Example only: 4.5%.</t>
         </r>
       </text>
     </comment>
@@ -1938,7 +1938,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Generally the standard is 3.15% a year after charges once retired (LifeGoals Standard set; Cautious 2.8%). Choose what you want to use. Example only: 3.15%.</t>
+          <t xml:space="preserve">Generally the standard is 3.15% a year after charges once retired (LifeMap Standard set; Cautious 2.8%). Choose what you want to use. Example only: 3.15%.</t>
         </r>
       </text>
     </comment>
@@ -4269,7 +4269,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3605" uniqueCount="1735">
   <si>
-    <t xml:space="preserve">LifeGoals calculators</t>
+    <t xml:space="preserve">LifeMap calculators</t>
   </si>
   <si>
     <t xml:space="preserve">Version 2.3 · 2 Oct 2026 · built from LifeGoals-Customer-Journey-Prototype.html (CALCS), corrected per the independent accuracy audit</t>
@@ -6459,13 +6459,13 @@
     <t xml:space="preserve">Pension growth after charges a year</t>
   </si>
   <si>
-    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use. Allowed: 1% to 7% · steps of 0.25%</t>
+    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 4.5% a year after charges while you work (LifeMap Standard set; Cautious 4%). Choose what you want to use. Allowed: 1% to 7% · steps of 0.25%</t>
   </si>
   <si>
     <t xml:space="preserve">Pay rises a year (contributions rise with pay)</t>
   </si>
   <si>
-    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 3% a year (Irish pay has grown about 3%–4% a year recently; LifeGoals Standard set). Choose what you want to use. Allowed: 0% to 6% · steps of 0.25%</t>
+    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 3% a year (Irish pay has grown about 3%–4% a year recently; LifeMap Standard set). Choose what you want to use. Allowed: 0% to 6% · steps of 0.25%</t>
   </si>
   <si>
     <t xml:space="preserve">Retirement savings target: × the yearly income you need</t>
@@ -6690,7 +6690,7 @@
     <t xml:space="preserve">Growth assumption a year</t>
   </si>
   <si>
-    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use. Allowed: 1% to 7% · steps of 0.5%</t>
+    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 4.5% a year after charges while you work (LifeMap Standard set; Cautious 4%). Choose what you want to use. Allowed: 1% to 7% · steps of 0.5%</t>
   </si>
   <si>
     <t xml:space="preserve">Your tax rate (0.2 = 20%, 0.4 = 40%)</t>
@@ -6915,7 +6915,7 @@
     <t xml:space="preserve">Growth assumption a year (once retired)</t>
   </si>
   <si>
-    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 3.15% a year after charges once retired (LifeGoals Standard set; Cautious 2.8%). Choose what you want to use. Allowed: 0% to 7% · steps of 0.05%</t>
+    <t xml:space="preserve">Type 3 · your choice · Generally the standard is 3.15% a year after charges once retired (LifeMap Standard set; Cautious 2.8%). Choose what you want to use. Allowed: 0% to 7% · steps of 0.05%</t>
   </si>
   <si>
     <t xml:space="preserve">Withdrawal taken at the</t>
@@ -9390,7 +9390,7 @@
     <t xml:space="preserve">https://eur-lex.europa.eu/eli/dir/2008/48/oj</t>
   </si>
   <si>
-    <t xml:space="preserve">STATEMENT READER RULES (product rules)  ·  LifeGoals product rule</t>
+    <t xml:space="preserve">STATEMENT READER RULES (product rules)  ·  LifeMap product rule</t>
   </si>
   <si>
     <t xml:space="preserve">Investment statement: shares at or above this = style 3 Growth  [Shares_For_Growth]</t>
@@ -9420,7 +9420,7 @@
     <t xml:space="preserve">Document reader spec</t>
   </si>
   <si>
-    <t xml:space="preserve">DISPLAY RULES AND STATISTICAL CONSTANTS  ·  LifeGoals product rule</t>
+    <t xml:space="preserve">DISPLAY RULES AND STATISTICAL CONSTANTS  ·  LifeMap product rule</t>
   </si>
   <si>
     <t xml:space="preserve">Show "Over 100 years" above this many months  [Cap_Months]</t>
@@ -9912,475 +9912,475 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="33" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="35" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="35" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -14874,11 +14874,11 @@
       <formula1>0</formula1>
       <formula2>500000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1% to 7% · steps of 0.25%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use.  Allowed: 1% to 7% · steps of 0.25%." promptTitle="Pension growth after charges a y" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C27" type="decimal">
+    <dataValidation allowBlank="true" error="Please enter 1% to 7% · steps of 0.25%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 4.5% a year after charges while you work (LifeMap Standard set; Cautious 4%). Choose what you want to use.  Allowed: 1% to 7% · steps of 0.25%." promptTitle="Pension growth after charges a y" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C27" type="decimal">
       <formula1>0.01</formula1>
       <formula2>0.07</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 6% · steps of 0.25%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 3% a year (Irish pay has grown about 3%–4% a year recently; LifeGoals Standard set). Choose what you want to use.  Allowed: 0% to 6% · steps of 0.25%." promptTitle="Pay rises a year (contributions " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C28" type="decimal">
+    <dataValidation allowBlank="true" error="Please enter 0% to 6% · steps of 0.25%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 3% a year (Irish pay has grown about 3%–4% a year recently; LifeMap Standard set). Choose what you want to use.  Allowed: 0% to 6% · steps of 0.25%." promptTitle="Pay rises a year (contributions " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C28" type="decimal">
       <formula1>0</formula1>
       <formula2>0.06</formula2>
     </dataValidation>
@@ -15576,7 +15576,7 @@
       <formula1>0</formula1>
       <formula2>0.025</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1% to 7% · steps of 0.5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use.  Allowed: 1% to 7% · steps of 0.5%." promptTitle="Growth assumption a year" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
+    <dataValidation allowBlank="true" error="Please enter 1% to 7% · steps of 0.5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 4.5% a year after charges while you work (LifeMap Standard set; Cautious 4%). Choose what you want to use.  Allowed: 1% to 7% · steps of 0.5%." promptTitle="Growth assumption a year" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
       <formula1>0.01</formula1>
       <formula2>0.07</formula2>
     </dataValidation>
@@ -16289,7 +16289,7 @@
       <formula1>0</formula1>
       <formula2>0.025</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1% to 7% · steps of 0.5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 4.5% a year after charges while you work (LifeGoals Standard set; Cautious 4%). Choose what you want to use.  Allowed: 1% to 7% · steps of 0.5%." promptTitle="Growth assumption a year" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
+    <dataValidation allowBlank="true" error="Please enter 1% to 7% · steps of 0.5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 4.5% a year after charges while you work (LifeMap Standard set; Cautious 4%). Choose what you want to use.  Allowed: 1% to 7% · steps of 0.5%." promptTitle="Growth assumption a year" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
       <formula1>0.01</formula1>
       <formula2>0.07</formula2>
     </dataValidation>
@@ -18144,7 +18144,7 @@
       <formula1>1000</formula1>
       <formula2>2000000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 7% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 3.15% a year after charges once retired (LifeGoals Standard set; Cautious 2.8%). Choose what you want to use.  Allowed: 0% to 7% · steps of 0.05%." promptTitle="Growth assumption a year (once r" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
+    <dataValidation allowBlank="true" error="Please enter 0% to 7% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 3.15% a year after charges once retired (LifeMap Standard set; Cautious 2.8%). Choose what you want to use.  Allowed: 0% to 7% · steps of 0.05%." promptTitle="Growth assumption a year (once r" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
       <formula1>0</formula1>
       <formula2>0.07</formula2>
     </dataValidation>
@@ -21854,6 +21854,10 @@
       <formula1>0</formula1>
       <formula2>0.03</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 0% to 8% · steps of 0.5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 5% a year before charges and tax for a mixed fund (long-run 5%–6% a year; Irish rules audit B3). Choose what you want to use.  Allowed: 0% to 8% · steps of 0.5%." promptTitle="Growth a year (before fees)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0.08</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €1,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €1,000,000." promptTitle="Monthly amount invested" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C11" type="decimal">
       <formula1>0</formula1>
       <formula2>1000000</formula2>
@@ -21861,10 +21865,6 @@
     <dataValidation allowBlank="true" error="Please enter €25 to €50,000 · steps of €25." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €25 to €50,000 · steps of €25." promptTitle="Monthly amount" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C16" type="decimal">
       <formula1>25</formula1>
       <formula2>50000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 8% · steps of 0.5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 5% a year before charges and tax for a mixed fund (long-run 5%–6% a year; Irish rules audit B3). Choose what you want to use.  Allowed: 0% to 8% · steps of 0.5%." promptTitle="Growth a year (before fees)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C18" type="decimal">
-      <formula1>0</formula1>
-      <formula2>0.08</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter Yes or No." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Optional: leave blank for none.  Allowed: Yes or No." promptTitle="Show in today's money?" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C20" type="list">
       <formula1>"Yes,No"</formula1>
@@ -22549,13 +22549,13 @@
     <mergeCell ref="B40:E40"/>
   </mergeCells>
   <dataValidations count="9">
+    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C13" type="whole">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €10,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between €2,500 and €3,500 for legal and survey fees (stamp duty is added for you). Enter your own figure.  Allowed: €0 to €10,000 · steps of €100." promptTitle="Legal and other buying fees" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C12" type="decimal">
       <formula1>0</formula1>
       <formula2>10000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C13" type="whole">
-      <formula1>1</formula1>
-      <formula2>30</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €15,000 to €2,500,000 · steps of €1,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure. In the app it is pre-filled from Your finances: income.  Allowed: €15,000 to €2,500,000 · steps of €1,000." promptTitle="Your gross yearly income" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C6" type="decimal">
       <formula1>15000</formula1>
@@ -35589,6 +35589,10 @@
     <mergeCell ref="B38:E38"/>
   </mergeCells>
   <dataValidations count="12">
+    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="whole">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €10,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between €2,500 and €3,500 for legal and survey fees (stamp duty is added for you). Enter your own figure.  Allowed: €0 to €10,000 · steps of €100." promptTitle="Legal and other buying fees" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C15" type="decimal">
       <formula1>0</formula1>
       <formula2>10000</formula2>
@@ -35596,10 +35600,6 @@
     <dataValidation allowBlank="true" error="Please enter €100,000 to €10,000,000 · steps of €5,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €100,000 to €10,000,000 · steps of €5,000." promptTitle="Home price" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="decimal">
       <formula1>100000</formula1>
       <formula2>10000000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="whole">
-      <formula1>1</formula1>
-      <formula2>30</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €500 to €50,000 · steps of €50." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €500 to €50,000 · steps of €50." promptTitle="Monthly rent" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C6" type="decimal">
       <formula1>500</formula1>

</xml_diff>

<commit_message>
Workbook C11 goal name 'Emergency fund'; spec §15: 'Enter 0' on euro fields only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhUEAkgdki1q9EpFqaquGU
</commit_message>
<xml_diff>
--- a/deliverables/LifeGoals-Calculators.xlsx
+++ b/deliverables/LifeGoals-Calculators.xlsx
@@ -6348,7 +6348,7 @@
     <t xml:space="preserve">• Spending must be at least €500, so there is no divide by zero.</t>
   </si>
   <si>
-    <t xml:space="preserve">ƒx  =IF(Still_To_Build&gt;0,"Safety net (plan kind safety: a reserve, not a spend)","No goal (cushion already in place)")</t>
+    <t xml:space="preserve">ƒx  =IF(Still_To_Build&gt;0,"Emergency fund (plan kind safety: a reserve, not a spend)","No goal (cushion already in place)")</t>
   </si>
   <si>
     <t xml:space="preserve">ƒx  =IF(Still_To_Build&gt;0,ROUND(Target,0),"—")</t>
@@ -9912,475 +9912,475 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="33" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="172" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="172" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="172" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="172" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="35" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="35" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="172" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="175" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -13628,7 +13628,7 @@
         <v>282</v>
       </c>
       <c r="C22" s="48" t="str">
-        <f aca="false">IF(Need_3&lt;&gt;"",Need_3,IF(Still_To_Build&gt;0,"Safety net (plan kind safety: a reserve, not a spend)","No goal (cushion already in place)"))</f>
+        <f aca="false">IF(Need_3&lt;&gt;"",Need_3,IF(Still_To_Build&gt;0,"Emergency fund (plan kind safety: a reserve, not a spend)","No goal (cushion already in place)"))</f>
         <v>Choose your essential monthly spending to see this</v>
       </c>
       <c r="E22" s="49" t="s">
@@ -14825,6 +14825,10 @@
     <dataValidation allowBlank="true" error="Please enter 0% to 5%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: %. Allowed: 0% to 5%." promptTitle="Annual charges % (if shown)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="decimal">
       <formula1>0</formula1>
       <formula2>0.05</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 0% to 2.5% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between 0.5% and 1.5% a year for pension charges (your statement shows yours). Enter your own figure.  Allowed: 0% to 2.5% · steps of 0.05%." promptTitle="Typical pension charges (if your" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C30" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0.025</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €50,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €50,000,000." promptTitle="Fund value today" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C11" type="decimal">
       <formula1>0</formula1>
@@ -14885,10 +14889,6 @@
     <dataValidation allowBlank="true" error="Please enter 20 to 33 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 25 times the yearly income you need (about 4% a year). Choose what you want to use.  Allowed: 20 to 33 · steps of 1." promptTitle="Retirement savings target: × the" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C29" type="whole">
       <formula1>20</formula1>
       <formula2>33</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 0% to 2.5% · steps of 0.05%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Usually between 0.5% and 1.5% a year for pension charges (your statement shows yours). Enter your own figure.  Allowed: 0% to 2.5% · steps of 0.05%." promptTitle="Typical pension charges (if your" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C30" type="decimal">
-      <formula1>0</formula1>
-      <formula2>0.025</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter 0% to 25% · steps of 1%." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 25% of the fund, the most allowed (first €200,000 tax-free, next €300,000 at 20%). Choose what you want to use.  Allowed: 0% to 25% · steps of 1%." promptTitle="Tax-free lump sum you plan to ta" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C31" type="decimal">
       <formula1>0</formula1>
@@ -25948,13 +25948,13 @@
       <formula1>0</formula1>
       <formula2>10000000</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter €0 to €50,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €50,000,000." promptTitle="Fund value today" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9" type="decimal">
+      <formula1>0</formula1>
+      <formula2>50000000</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €100,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €100,000,000." promptTitle="Total value" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C10" type="decimal">
       <formula1>0</formula1>
       <formula2>100000000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter €0 to €50,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €50,000,000." promptTitle="Fund value today" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9" type="decimal">
-      <formula1>0</formula1>
-      <formula2>50000000</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €100,000,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Unit: €. Allowed: €0 to €100,000,000." promptTitle="Property value (valuation)" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C8" type="decimal">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
Copy pass (journey-spec §20): plain-human UI text
- 26 customer-facing blocks reworded in the prototype (accuracy fixes where
  §17 to §19 left old wording, passive to active, contractions, trimmed
  restated headings, one run-on split); 4 README lines in the workbook.
- Words only: no code, markup, IDs, logic or numbers changed. Protected
  copy, gates, example cards, sources, dates and calculator result lines
  untouched.
- docs/copy-audit.md lists every change in the Agent Handoff Audit /
  Optimized Presentation Layer format, what was left alone and why.
- Suite green: e2e x3, choices, s19, check17, check16, a11y, calc-vs-xlsx
  145/145, recalc 0 errors.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhUEAkgdki1q9EpFqaquGU
</commit_message>
<xml_diff>
--- a/deliverables/LifeGoals-Calculators.xlsx
+++ b/deliverables/LifeGoals-Calculators.xlsx
@@ -4421,16 +4421,16 @@
     <t xml:space="preserve">• Open a calculator from the list below. Fill the yellow cells (blue text): everything else updates on its own.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Every number is one of three types (journey spec §14). Type 1, set by Government (tax, USC, PRSI, relief %, lump-sum bands, DIRT, exit tax, Central Bank limits, full State Pension and benefit rates): on the Assumptions sheet, not an input. Type 2, varies within a known range (mortgage rate, card APR, fund charges, the State Pension you will get …): a yellow input with "Usually between X and Y (source)". Type 3, personal (inflation, growth, pay rises, emergency months, drawdown timing, retirement multiple, and your own figures): a yellow input left BLANK with "Generally the standard is X (source). Choose what you want to use." Retirement age and plan-until age are blank with guidance only, never a standard.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Blank inputs stay blank: results that need them show "Choose your … to see this". Switch "Fill example values?" (above) to Yes to fill every blank input with its grey "Example only" figure (the standard, or the sample customer's figure).</t>
+    <t xml:space="preserve">• Every number is one of three types (journey spec §14, §18). Type 1, set by Government (tax, USC, PRSI, relief %, lump-sum bands, DIRT, exit tax, Central Bank limits, full State Pension and benefit rates): on the Assumptions sheet, not an input. Type 2, a market rate or a figure you enter yourself (mortgage rate, card APR, fund charges, the State Pension you will get …): a yellow input with a suggested figure and its source, or "Usually between X and Y (source)" where an official range exists. Type 3, personal (inflation, growth, pay rises, emergency months, drawdown timing, retirement multiple, and your own figures): a yellow input left BLANK with "Generally the standard is X (source). Choose what you want to use." Retirement age and plan-until age are blank with guidance only, never a standard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Blank inputs stay blank: results that need them show "Choose your … to see this". Set "Fill example values?" (above) to Yes to fill every blank input with its grey "Example only" figure (the standard, or the sample customer's figure).</t>
   </si>
   <si>
     <t xml:space="preserve">• Each input cell shows its unit and allowed range when you click it, and refuses values outside it. The default is in the cell note and at the far right.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Market rates (mortgage, loans, cards, deposits, buying fees, fund charges) are never pre-filled. Beside each one is a suggested rate with its source, from the Partner rates block on the Assumptions sheet: by default Central Bank of Ireland averages with their month (journey spec §18). A partner can put its own rates and name there ("Suggested by …"). Law values cannot be changed.</t>
+    <t xml:space="preserve">• Market rates (mortgage, loans, cards, deposits, buying fees, fund charges) are never pre-filled. Beside each is a suggested rate with its source, from the Settings sheet: by default Central Bank of Ireland averages with their month (journey spec §18, §19). A partner can put its own rates and name there ("Suggested by …"). Law values cannot be changed.</t>
   </si>
   <si>
     <t xml:space="preserve">• Facts and law (tax bands, State rates, Central Bank rules, stamp duty, lump-sum bands …) are on the Assumptions sheet, the Irish rules register (Irish rules 2026 · checked 2 Oct 2026). Take-home pay is worked out on the Tax engine sheet, which C25 and C26 use.</t>
@@ -4442,7 +4442,7 @@
     <t xml:space="preserve">• Inflation is the client's own choice: the yellow "Inflation you expect" cell on each calculator that uses it starts blank. While it is blank, results that need it say "Choose your inflation rate to see this"; 0% is a real choice (no adjustment for prices).</t>
   </si>
   <si>
-    <t xml:space="preserve">• Statements: grey-blue cells under "FROM YOUR STATEMENT" are filled by the document reader. The FIGURE USED box applies the rule statement figure if present, else your typed figure, and says which was used. See the "Document reader spec" sheet.</t>
+    <t xml:space="preserve">• Statements: grey-blue cells under "FROM YOUR STATEMENT" are filled by the document reader. The FIGURE USED box uses the statement figure if there is one, otherwise your typed figure, and says which. See the "Document reader spec" sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">• The workbook recalculates automatically, including when it is opened.</t>
@@ -38542,13 +38542,13 @@
       <formula1>0</formula1>
       <formula2>10000</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="whole">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €100,000 to €10,000,000 · steps of €5,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €100,000 to €10,000,000 · steps of €5,000." promptTitle="Home price" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="decimal">
       <formula1>100000</formula1>
       <formula2>10000000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="whole">
-      <formula1>1</formula1>
-      <formula2>30</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €500 to €50,000 · steps of €50." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €500 to €50,000 · steps of €50." promptTitle="Monthly rent" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C6" type="decimal">
       <formula1>500</formula1>

</xml_diff>

<commit_message>
Prototype §23 and §24: Emergency fund naming, real cover photo, Budget 2027 note, Liabilities mortgage first, What-if clarity, saving files via downloads
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhUEAkgdki1q9EpFqaquGU
</commit_message>
<xml_diff>
--- a/deliverables/LifeGoals-Calculators.xlsx
+++ b/deliverables/LifeGoals-Calculators.xlsx
@@ -4571,7 +4571,7 @@
     <t xml:space="preserve">C11</t>
   </si>
   <si>
-    <t xml:space="preserve">How strong is my financial cushion?</t>
+    <t xml:space="preserve">How strong is my emergency fund?</t>
   </si>
   <si>
     <t xml:space="preserve">C12</t>
@@ -6407,7 +6407,7 @@
     <t xml:space="preserve">Category: Savings &amp; Goals · prototype id: emergency</t>
   </si>
   <si>
-    <t xml:space="preserve">Question it answers: How strong is my financial cushion?</t>
+    <t xml:space="preserve">Question it answers: How strong is my emergency fund?</t>
   </si>
   <si>
     <t xml:space="preserve">Shows how many months of essential spending your easy-access savings cover, against your target.</t>
@@ -6419,7 +6419,7 @@
     <t xml:space="preserve">Type 3 · your figure · Your own figure. In the app it is pre-filled from Your finances: costs + mortgage + debt repayments. Allowed: €500 to €100,000 · steps of €100</t>
   </si>
   <si>
-    <t xml:space="preserve">Safety net: months of essential spending</t>
+    <t xml:space="preserve">Emergency fund: months of essential spending</t>
   </si>
   <si>
     <t xml:space="preserve">months</t>
@@ -6428,7 +6428,7 @@
     <t xml:space="preserve">Type 3 · your choice · Generally the standard is 6 months of essential spending (3 if you have two secure incomes). Choose what you want to use. Allowed: 3 to 12 · steps of 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Build the safety net within (years, for the plan)</t>
+    <t xml:space="preserve">Build the emergency fund within (years, for the plan)</t>
   </si>
   <si>
     <t xml:space="preserve">Type 3 · your figure · Your own figure. Allowed: 1 to 10 · steps of 1</t>
@@ -6446,7 +6446,7 @@
     <t xml:space="preserve">ƒx  =Savings/Essential_Spending</t>
   </si>
   <si>
-    <t xml:space="preserve">Target cushion</t>
+    <t xml:space="preserve">Target emergency fund</t>
   </si>
   <si>
     <t xml:space="preserve">ƒx  =Essential_Spending*Months_Wanted</t>
@@ -6464,7 +6464,7 @@
     <t xml:space="preserve">• Spending must be at least €500, so there is no divide by zero.</t>
   </si>
   <si>
-    <t xml:space="preserve">ƒx  =IF(Still_To_Build&gt;0,"Emergency fund (plan kind safety: a reserve, not a spend)","No goal (cushion already in place)")</t>
+    <t xml:space="preserve">ƒx  =IF(Still_To_Build&gt;0,"Emergency fund (plan kind safety: a reserve, not a spend)","No goal (emergency fund already in place)")</t>
   </si>
   <si>
     <t xml:space="preserve">ƒx  =IF(Still_To_Build&gt;0,ROUND(Target,0),"—")</t>
@@ -6488,7 +6488,7 @@
     <t xml:space="preserve">Needs: easy-access savings</t>
   </si>
   <si>
-    <t xml:space="preserve">Needs: years to build the safety net</t>
+    <t xml:space="preserve">Needs: years to build the emergency fund</t>
   </si>
   <si>
     <t xml:space="preserve">C12 · Retirement projection</t>
@@ -14669,7 +14669,7 @@
         <v>281</v>
       </c>
       <c r="C22" s="48" t="str">
-        <f aca="false">IF(Need_3&lt;&gt;"",Need_3,IF(Still_To_Build&gt;0,"Emergency fund (plan kind safety: a reserve, not a spend)","No goal (cushion already in place)"))</f>
+        <f aca="false">IF(Need_3&lt;&gt;"",Need_3,IF(Still_To_Build&gt;0,"Emergency fund (plan kind safety: a reserve, not a spend)","No goal (emergency fund already in place)"))</f>
         <v>Choose your essential monthly spending to see this</v>
       </c>
       <c r="E22" s="49" t="s">
@@ -14706,7 +14706,7 @@
       </c>
       <c r="C25" s="51" t="str">
         <f aca="false">IF(Need_5&lt;&gt;"",Need_5,Safety_Goal_Years)</f>
-        <v>Choose your years to build the safety net to see this</v>
+        <v>Choose your years to build the emergency fund to see this</v>
       </c>
       <c r="E25" s="49" t="s">
         <v>691</v>
@@ -14763,8 +14763,8 @@
         <v>696</v>
       </c>
       <c r="C32" s="52" t="str">
-        <f aca="false">IF(Safety_Goal_Years="","Choose your years to build the safety net to see this","")</f>
-        <v>Choose your years to build the safety net to see this</v>
+        <f aca="false">IF(Safety_Goal_Years="","Choose your years to build the emergency fund to see this","")</f>
+        <v>Choose your years to build the emergency fund to see this</v>
       </c>
     </row>
   </sheetData>
@@ -14778,11 +14778,11 @@
       <formula1>500</formula1>
       <formula2>100000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 3 to 12 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 6 months of essential spending (3 if you have two secure incomes). Choose what you want to use.  Allowed: 3 to 12 · steps of 1." promptTitle="Safety net: months of essential " showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="whole">
+    <dataValidation allowBlank="true" error="Please enter 3 to 12 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Generally the standard is 6 months of essential spending (3 if you have two secure incomes). Choose what you want to use.  Allowed: 3 to 12 · steps of 1." promptTitle="Emergency fund: months" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="whole">
       <formula1>3</formula1>
       <formula2>12</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1 to 10 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 10 · steps of 1." promptTitle="Build the safety net within (yea" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C8" type="whole">
+    <dataValidation allowBlank="true" error="Please enter 1 to 10 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 10 · steps of 1." promptTitle="Build the emergency fund within" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C8" type="whole">
       <formula1>1</formula1>
       <formula2>10</formula2>
     </dataValidation>
@@ -23602,13 +23602,13 @@
     <mergeCell ref="B40:E40"/>
   </mergeCells>
   <dataValidations count="9">
+    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C13" type="whole">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €10,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Optional: your own legal and survey fees. No published figure, so no suggestion unless a partner sets one. Leave blank to count €0. Allowed: €0 to €10,000 · steps of €100" promptTitle="Legal and other buying fees" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C12" type="decimal">
       <formula1>0</formula1>
       <formula2>10000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C13" type="whole">
-      <formula1>1</formula1>
-      <formula2>30</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €15,000 to €2,500,000 · steps of €1,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure. In the app it is pre-filled from Your finances: income.  Allowed: €15,000 to €2,500,000 · steps of €1,000." promptTitle="Your gross yearly income" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C6" type="decimal">
       <formula1>15000</formula1>
@@ -38538,13 +38538,13 @@
     <mergeCell ref="B38:E38"/>
   </mergeCells>
   <dataValidations count="12">
+    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="whole">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €0 to €10,000 · steps of €100." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Optional: your own legal and survey fees. No published figure, so no suggestion unless a partner sets one. Leave blank to count €0. Allowed: €0 to €10,000 · steps of €100" promptTitle="Legal and other buying fees" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C15" type="decimal">
       <formula1>0</formula1>
       <formula2>10000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter 1 to 30 · steps of 1." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: 1 to 30 · steps of 1." promptTitle="Years until you buy (for the pla" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C17" type="whole">
-      <formula1>1</formula1>
-      <formula2>30</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Please enter €100,000 to €10,000,000 · steps of €5,000." errorStyle="stop" errorTitle="Outside the allowed range" operator="between" prompt="Your own figure.  Allowed: €100,000 to €10,000,000 · steps of €5,000." promptTitle="Home price" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7" type="decimal">
       <formula1>100000</formula1>

</xml_diff>

<commit_message>
Standards card lists only the true remainder; workbook Set_inv label/charges match the app
Card compares by key (15 standards applied, 3 left to the customer);
Set_inv_Label built from the same inputs; override test (4 cases, 12 checks)
compares app and workbook exactly. sfix 40/40, overridetest 12/12,
calc-vs-xlsx 145/145, recalc 0 errors, no formula without cached value.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhUEAkgdki1q9EpFqaquGU
</commit_message>
<xml_diff>
--- a/deliverables/LifeGoals-Calculators.xlsx
+++ b/deliverables/LifeGoals-Calculators.xlsx
@@ -4398,7 +4398,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3935" uniqueCount="1988">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3934" uniqueCount="1987">
   <si>
     <t xml:space="preserve">LifeMap calculators</t>
   </si>
@@ -9282,9 +9282,6 @@
   </si>
   <si>
     <t xml:space="preserve">Investments grow (a year, after charges and tax)  [Set_inv]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a planning assumption, not a forecast: derived from the growth before fees and tax (Set_invGross), the charges (Suggest_Fund_Charges) and the exit tax every 8 years (Exit_Tax, Deemed_Disposal_Years). Edit those, not this cell.</t>
   </si>
   <si>
     <t xml:space="preserve">Derived: the growth before fees and tax (above), the charges (Market rates) and the exit tax and 8-year rule (Tax rules)</t>
@@ -32133,17 +32130,18 @@
         <f aca="false">ROUND(((1+Set_invGross-0.01-IF(ISNUMBER(Suggest_Fund_Charges),Suggest_Fund_Charges,0.01))^Deemed_Disposal_Years-Exit_Tax*((1+Set_invGross-0.01-IF(ISNUMBER(Suggest_Fund_Charges),Suggest_Fund_Charges,0.01))^Deemed_Disposal_Years-1))^(1/Deemed_Disposal_Years)-1,3)</f>
         <v>0.019</v>
       </c>
-      <c r="G11" s="107" t="s">
+      <c r="G11" s="107" t="str">
+        <f aca="false">"a planning assumption, not a prediction: "&amp;ROUND(Set_invGross*1000,0)/10&amp;"% before fees and tax, less about "&amp;ROUND(IF(ISNUMBER(Suggest_Fund_Charges),Suggest_Fund_Charges,0.01)*1000,0)/10&amp;"% charges, less "&amp;ROUND(Exit_Tax*100,0)&amp;"% exit tax taken every "&amp;Deemed_Disposal_Years&amp;" years"</f>
+        <v>a planning assumption, not a prediction: 5% before fees and tax, less about 1% charges, less 38% exit tax taken every 8 years</v>
+      </c>
+      <c r="H11" s="116" t="s">
         <v>1628</v>
-      </c>
-      <c r="H11" s="116" t="s">
-        <v>1629</v>
       </c>
       <c r="I11" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J11" s="116" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
       <c r="K11" s="116" t="s">
         <v>1617</v>
@@ -32151,22 +32149,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="1" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="C12" s="109" t="n">
         <v>0.05</v>
       </c>
       <c r="G12" s="107" t="s">
+        <v>1631</v>
+      </c>
+      <c r="H12" s="116" t="s">
         <v>1632</v>
-      </c>
-      <c r="H12" s="116" t="s">
-        <v>1633</v>
       </c>
       <c r="I12" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J12" s="116" t="s">
-        <v>1634</v>
+        <v>1633</v>
       </c>
       <c r="K12" s="116" t="s">
         <v>1617</v>
@@ -32174,7 +32172,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="1" t="s">
-        <v>1635</v>
+        <v>1634</v>
       </c>
       <c r="C13" s="109" t="n">
         <v>0.045</v>
@@ -32183,16 +32181,16 @@
         <v>0.04</v>
       </c>
       <c r="G13" s="107" t="s">
+        <v>1635</v>
+      </c>
+      <c r="H13" s="116" t="s">
         <v>1636</v>
-      </c>
-      <c r="H13" s="116" t="s">
-        <v>1637</v>
       </c>
       <c r="I13" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J13" s="116" t="s">
-        <v>1638</v>
+        <v>1637</v>
       </c>
       <c r="K13" s="116" t="s">
         <v>1617</v>
@@ -32200,7 +32198,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="1" t="s">
-        <v>1639</v>
+        <v>1638</v>
       </c>
       <c r="C14" s="109" t="n">
         <v>0.0315</v>
@@ -32209,16 +32207,16 @@
         <v>0.028</v>
       </c>
       <c r="G14" s="107" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="H14" s="116" t="s">
-        <v>1637</v>
+        <v>1636</v>
       </c>
       <c r="I14" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J14" s="116" t="s">
-        <v>1641</v>
+        <v>1640</v>
       </c>
       <c r="K14" s="116" t="s">
         <v>1617</v>
@@ -32226,306 +32224,306 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="115" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="1" t="s">
-        <v>1643</v>
+        <v>1642</v>
       </c>
       <c r="C16" s="109" t="n">
         <v>0.03</v>
       </c>
       <c r="G16" s="107" t="s">
+        <v>1643</v>
+      </c>
+      <c r="H16" s="116" t="s">
         <v>1644</v>
-      </c>
-      <c r="H16" s="116" t="s">
-        <v>1645</v>
       </c>
       <c r="I16" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J16" s="116" t="s">
+        <v>1645</v>
+      </c>
+      <c r="K16" s="116" t="s">
         <v>1646</v>
-      </c>
-      <c r="K16" s="116" t="s">
-        <v>1647</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>1648</v>
+        <v>1647</v>
       </c>
       <c r="C17" s="109" t="n">
         <v>0.02</v>
       </c>
       <c r="G17" s="107" t="s">
+        <v>1648</v>
+      </c>
+      <c r="H17" s="116" t="s">
         <v>1649</v>
-      </c>
-      <c r="H17" s="116" t="s">
-        <v>1650</v>
       </c>
       <c r="I17" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J17" s="116" t="s">
-        <v>1651</v>
+        <v>1650</v>
       </c>
       <c r="K17" s="116" t="s">
-        <v>1647</v>
+        <v>1646</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="C18" s="109" t="n">
         <v>0.01</v>
       </c>
       <c r="G18" s="107" t="s">
+        <v>1652</v>
+      </c>
+      <c r="H18" s="116" t="s">
         <v>1653</v>
-      </c>
-      <c r="H18" s="116" t="s">
-        <v>1654</v>
       </c>
       <c r="I18" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J18" s="116"/>
       <c r="K18" s="116" t="s">
-        <v>1647</v>
+        <v>1646</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="115" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="1" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="C20" s="109" t="n">
         <v>0.5</v>
       </c>
       <c r="G20" s="107" t="s">
+        <v>1656</v>
+      </c>
+      <c r="H20" s="116" t="s">
         <v>1657</v>
-      </c>
-      <c r="H20" s="116" t="s">
-        <v>1658</v>
       </c>
       <c r="I20" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J20" s="116" t="s">
+        <v>1658</v>
+      </c>
+      <c r="K20" s="116" t="s">
         <v>1659</v>
-      </c>
-      <c r="K20" s="116" t="s">
-        <v>1660</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="1" t="s">
-        <v>1661</v>
+        <v>1660</v>
       </c>
       <c r="C21" s="107" t="n">
         <v>25</v>
       </c>
       <c r="G21" s="107" t="s">
+        <v>1661</v>
+      </c>
+      <c r="H21" s="116" t="s">
         <v>1662</v>
-      </c>
-      <c r="H21" s="116" t="s">
-        <v>1663</v>
       </c>
       <c r="I21" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J21" s="116" t="s">
+        <v>1663</v>
+      </c>
+      <c r="K21" s="116" t="s">
         <v>1664</v>
-      </c>
-      <c r="K21" s="116" t="s">
-        <v>1665</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>1666</v>
+        <v>1665</v>
       </c>
       <c r="C22" s="109" t="n">
         <v>0.8</v>
       </c>
       <c r="G22" s="107" t="s">
+        <v>1666</v>
+      </c>
+      <c r="H22" s="116" t="s">
         <v>1667</v>
-      </c>
-      <c r="H22" s="116" t="s">
-        <v>1668</v>
       </c>
       <c r="I22" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J22" s="116"/>
       <c r="K22" s="116" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="1" t="s">
-        <v>1669</v>
+        <v>1668</v>
       </c>
       <c r="C23" s="109" t="n">
         <v>0.25</v>
       </c>
       <c r="G23" s="107" t="s">
+        <v>1669</v>
+      </c>
+      <c r="H23" s="116" t="s">
         <v>1670</v>
       </c>
-      <c r="H23" s="116" t="s">
+      <c r="I23" s="116" t="s">
         <v>1671</v>
-      </c>
-      <c r="I23" s="116" t="s">
-        <v>1672</v>
       </c>
       <c r="J23" s="116"/>
       <c r="K23" s="116" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="115" t="s">
-        <v>1673</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="1" t="s">
-        <v>1674</v>
+        <v>1673</v>
       </c>
       <c r="C25" s="107" t="n">
         <v>6</v>
       </c>
       <c r="G25" s="107" t="s">
+        <v>1674</v>
+      </c>
+      <c r="H25" s="116" t="s">
         <v>1675</v>
-      </c>
-      <c r="H25" s="116" t="s">
-        <v>1676</v>
       </c>
       <c r="I25" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J25" s="116" t="s">
+        <v>1676</v>
+      </c>
+      <c r="K25" s="116" t="s">
         <v>1677</v>
-      </c>
-      <c r="K25" s="116" t="s">
-        <v>1678</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="1" t="s">
-        <v>1679</v>
+        <v>1678</v>
       </c>
       <c r="C26" s="107" t="n">
         <v>3</v>
       </c>
       <c r="G26" s="107" t="s">
+        <v>1679</v>
+      </c>
+      <c r="H26" s="116" t="s">
         <v>1680</v>
-      </c>
-      <c r="H26" s="116" t="s">
-        <v>1681</v>
       </c>
       <c r="I26" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J26" s="116"/>
       <c r="K26" s="116" t="s">
-        <v>1678</v>
+        <v>1677</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="1" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="C27" s="107" t="n">
         <v>5</v>
       </c>
       <c r="G27" s="107" t="s">
+        <v>1682</v>
+      </c>
+      <c r="H27" s="116" t="s">
         <v>1683</v>
-      </c>
-      <c r="H27" s="116" t="s">
-        <v>1684</v>
       </c>
       <c r="I27" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J27" s="116" t="s">
+        <v>1684</v>
+      </c>
+      <c r="K27" s="116" t="s">
         <v>1685</v>
-      </c>
-      <c r="K27" s="116" t="s">
-        <v>1686</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="1" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="C28" s="109" t="n">
         <v>0.4</v>
       </c>
       <c r="G28" s="107" t="s">
+        <v>1687</v>
+      </c>
+      <c r="H28" s="116" t="s">
         <v>1688</v>
-      </c>
-      <c r="H28" s="116" t="s">
-        <v>1689</v>
       </c>
       <c r="I28" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J28" s="116"/>
       <c r="K28" s="116" t="s">
-        <v>1690</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="1" t="s">
-        <v>1691</v>
+        <v>1690</v>
       </c>
       <c r="C29" s="109" t="n">
         <v>0.5</v>
       </c>
       <c r="G29" s="107" t="s">
+        <v>1691</v>
+      </c>
+      <c r="H29" s="116" t="s">
         <v>1692</v>
-      </c>
-      <c r="H29" s="116" t="s">
-        <v>1693</v>
       </c>
       <c r="I29" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J29" s="116" t="s">
-        <v>1694</v>
+        <v>1693</v>
       </c>
       <c r="K29" s="116" t="s">
-        <v>1690</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="1" t="s">
-        <v>1695</v>
+        <v>1694</v>
       </c>
       <c r="C30" s="108" t="n">
         <v>300</v>
       </c>
       <c r="G30" s="107" t="s">
-        <v>1696</v>
+        <v>1695</v>
       </c>
       <c r="H30" s="116" t="s">
-        <v>1693</v>
+        <v>1692</v>
       </c>
       <c r="I30" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J30" s="116" t="s">
+        <v>1696</v>
+      </c>
+      <c r="K30" s="116" t="s">
         <v>1697</v>
-      </c>
-      <c r="K30" s="116" t="s">
-        <v>1698</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32535,54 +32533,54 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="1" t="s">
-        <v>1699</v>
+        <v>1698</v>
       </c>
       <c r="C32" s="109" t="n">
         <v>0.6</v>
       </c>
       <c r="G32" s="107" t="s">
+        <v>1699</v>
+      </c>
+      <c r="H32" s="116" t="s">
         <v>1700</v>
-      </c>
-      <c r="H32" s="116" t="s">
-        <v>1701</v>
       </c>
       <c r="I32" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J32" s="116"/>
       <c r="K32" s="116" t="s">
-        <v>1702</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="1" t="s">
-        <v>1703</v>
+        <v>1702</v>
       </c>
       <c r="C33" s="107" t="n">
         <v>15</v>
       </c>
       <c r="G33" s="107" t="s">
-        <v>1704</v>
+        <v>1703</v>
       </c>
       <c r="H33" s="116" t="s">
-        <v>1701</v>
+        <v>1700</v>
       </c>
       <c r="I33" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J33" s="116"/>
       <c r="K33" s="116" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="115" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="1" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="C35" s="118" t="n">
         <v>0.02</v>
@@ -32594,24 +32592,24 @@
         <v>0.06</v>
       </c>
       <c r="G35" s="107" t="s">
+        <v>1707</v>
+      </c>
+      <c r="H35" s="116" t="s">
         <v>1708</v>
-      </c>
-      <c r="H35" s="116" t="s">
-        <v>1709</v>
       </c>
       <c r="I35" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J35" s="116" t="s">
+        <v>1709</v>
+      </c>
+      <c r="K35" s="116" t="s">
         <v>1710</v>
-      </c>
-      <c r="K35" s="116" t="s">
-        <v>1711</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="1" t="s">
-        <v>1712</v>
+        <v>1711</v>
       </c>
       <c r="C36" s="118" t="n">
         <v>0.05</v>
@@ -32623,24 +32621,24 @@
         <v>0.16</v>
       </c>
       <c r="G36" s="107" t="s">
+        <v>1707</v>
+      </c>
+      <c r="H36" s="116" t="s">
         <v>1708</v>
-      </c>
-      <c r="H36" s="116" t="s">
-        <v>1709</v>
       </c>
       <c r="I36" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J36" s="116" t="s">
-        <v>1713</v>
+        <v>1712</v>
       </c>
       <c r="K36" s="116" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="1" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
       <c r="C37" s="118" t="n">
         <v>0.5</v>
@@ -32652,181 +32650,181 @@
         <v>0.2</v>
       </c>
       <c r="G37" s="107" t="s">
+        <v>1714</v>
+      </c>
+      <c r="H37" s="116" t="s">
         <v>1715</v>
-      </c>
-      <c r="H37" s="116" t="s">
-        <v>1716</v>
       </c>
       <c r="I37" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J37" s="116"/>
       <c r="K37" s="116" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="115" t="s">
-        <v>1717</v>
+        <v>1716</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="1" t="s">
+        <v>1717</v>
+      </c>
+      <c r="C39" s="107" t="s">
         <v>1718</v>
       </c>
-      <c r="C39" s="107" t="s">
+      <c r="G39" s="107" t="s">
         <v>1719</v>
       </c>
-      <c r="G39" s="107" t="s">
+      <c r="H39" s="116" t="s">
         <v>1720</v>
-      </c>
-      <c r="H39" s="116" t="s">
-        <v>1721</v>
       </c>
       <c r="I39" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J39" s="116" t="s">
+        <v>1721</v>
+      </c>
+      <c r="K39" s="116" t="s">
         <v>1722</v>
-      </c>
-      <c r="K39" s="116" t="s">
-        <v>1723</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="1" t="s">
+        <v>1723</v>
+      </c>
+      <c r="C40" s="107" t="s">
+        <v>1718</v>
+      </c>
+      <c r="G40" s="107" t="s">
         <v>1724</v>
       </c>
-      <c r="C40" s="107" t="s">
-        <v>1719</v>
-      </c>
-      <c r="G40" s="107" t="s">
+      <c r="H40" s="116" t="s">
         <v>1725</v>
-      </c>
-      <c r="H40" s="116" t="s">
-        <v>1726</v>
       </c>
       <c r="I40" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J40" s="116" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="K40" s="116" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="1" t="s">
+        <v>1727</v>
+      </c>
+      <c r="C41" s="107" t="s">
         <v>1728</v>
       </c>
-      <c r="C41" s="107" t="s">
+      <c r="G41" s="107" t="s">
         <v>1729</v>
       </c>
-      <c r="G41" s="107" t="s">
+      <c r="H41" s="116" t="s">
         <v>1730</v>
-      </c>
-      <c r="H41" s="116" t="s">
-        <v>1731</v>
       </c>
       <c r="I41" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J41" s="116"/>
       <c r="K41" s="116" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="1" t="s">
+        <v>1731</v>
+      </c>
+      <c r="C42" s="107" t="s">
         <v>1732</v>
       </c>
-      <c r="C42" s="107" t="s">
+      <c r="G42" s="107" t="s">
         <v>1733</v>
       </c>
-      <c r="G42" s="107" t="s">
+      <c r="H42" s="116" t="s">
         <v>1734</v>
-      </c>
-      <c r="H42" s="116" t="s">
-        <v>1735</v>
       </c>
       <c r="I42" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J42" s="116"/>
       <c r="K42" s="116" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="1" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="C43" s="107" t="n">
         <v>5</v>
       </c>
       <c r="G43" s="107" t="s">
+        <v>1736</v>
+      </c>
+      <c r="H43" s="116" t="s">
         <v>1737</v>
-      </c>
-      <c r="H43" s="116" t="s">
-        <v>1738</v>
       </c>
       <c r="I43" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J43" s="116"/>
       <c r="K43" s="116" t="s">
-        <v>1739</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="1" t="s">
-        <v>1740</v>
+        <v>1739</v>
       </c>
       <c r="C44" s="107" t="n">
         <v>2</v>
       </c>
       <c r="G44" s="107" t="s">
+        <v>1740</v>
+      </c>
+      <c r="H44" s="116" t="s">
         <v>1741</v>
-      </c>
-      <c r="H44" s="116" t="s">
-        <v>1742</v>
       </c>
       <c r="I44" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J44" s="116"/>
       <c r="K44" s="116" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="115" t="s">
-        <v>1744</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="1" t="s">
-        <v>1745</v>
+        <v>1744</v>
       </c>
       <c r="C46" s="109" t="n">
         <v>0.0348</v>
       </c>
       <c r="D46" s="109"/>
       <c r="G46" s="107" t="s">
+        <v>1745</v>
+      </c>
+      <c r="H46" s="116" t="s">
         <v>1746</v>
       </c>
-      <c r="H46" s="116" t="s">
+      <c r="I46" s="116" t="s">
         <v>1747</v>
       </c>
-      <c r="I46" s="116" t="s">
+      <c r="J46" s="116" t="s">
         <v>1748</v>
       </c>
-      <c r="J46" s="116" t="s">
+      <c r="K46" s="116" t="s">
         <v>1749</v>
-      </c>
-      <c r="K46" s="116" t="s">
-        <v>1750</v>
       </c>
       <c r="L46" s="116" t="str">
         <f aca="false">IF(D46&lt;&gt;"","Suggested by "&amp;IF(Partner_Name="","your provider",Partner_Name),G46)</f>
@@ -32839,26 +32837,26 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="1" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="C47" s="109" t="n">
         <v>0.0672</v>
       </c>
       <c r="D47" s="109"/>
       <c r="G47" s="107" t="s">
+        <v>1751</v>
+      </c>
+      <c r="H47" s="116" t="s">
+        <v>1746</v>
+      </c>
+      <c r="I47" s="116" t="s">
+        <v>1747</v>
+      </c>
+      <c r="J47" s="116" t="s">
         <v>1752</v>
       </c>
-      <c r="H47" s="116" t="s">
-        <v>1747</v>
-      </c>
-      <c r="I47" s="116" t="s">
-        <v>1748</v>
-      </c>
-      <c r="J47" s="116" t="s">
-        <v>1753</v>
-      </c>
       <c r="K47" s="116" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="L47" s="116" t="str">
         <f aca="false">IF(D47&lt;&gt;"","Suggested by "&amp;IF(Partner_Name="","your provider",Partner_Name),G47)</f>
@@ -32871,24 +32869,24 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="1" t="s">
-        <v>1754</v>
+        <v>1753</v>
       </c>
       <c r="C48" s="109"/>
       <c r="D48" s="109"/>
       <c r="G48" s="107" t="s">
+        <v>1754</v>
+      </c>
+      <c r="H48" s="116" t="s">
+        <v>1746</v>
+      </c>
+      <c r="I48" s="116" t="s">
         <v>1755</v>
       </c>
-      <c r="H48" s="116" t="s">
-        <v>1747</v>
-      </c>
-      <c r="I48" s="116" t="s">
+      <c r="J48" s="116" t="s">
         <v>1756</v>
       </c>
-      <c r="J48" s="116" t="s">
-        <v>1757</v>
-      </c>
       <c r="K48" s="116" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="L48" s="116" t="str">
         <f aca="false">IF(D48&lt;&gt;"","Suggested by "&amp;IF(Partner_Name="","your provider",Partner_Name),G48)</f>
@@ -32901,26 +32899,26 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="1" t="s">
-        <v>1758</v>
+        <v>1757</v>
       </c>
       <c r="C49" s="109" t="n">
         <v>0.0192</v>
       </c>
       <c r="D49" s="109"/>
       <c r="G49" s="107" t="s">
+        <v>1758</v>
+      </c>
+      <c r="H49" s="116" t="s">
+        <v>1746</v>
+      </c>
+      <c r="I49" s="116" t="s">
+        <v>1747</v>
+      </c>
+      <c r="J49" s="116" t="s">
         <v>1759</v>
       </c>
-      <c r="H49" s="116" t="s">
-        <v>1747</v>
-      </c>
-      <c r="I49" s="116" t="s">
-        <v>1748</v>
-      </c>
-      <c r="J49" s="116" t="s">
-        <v>1760</v>
-      </c>
       <c r="K49" s="116" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="L49" s="116" t="str">
         <f aca="false">IF(D49&lt;&gt;"","Suggested by "&amp;IF(Partner_Name="","your provider",Partner_Name),G49)</f>
@@ -32933,22 +32931,22 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="1" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="C50" s="108"/>
       <c r="D50" s="108"/>
       <c r="G50" s="107" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="H50" s="116" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="I50" s="116" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="J50" s="116"/>
       <c r="K50" s="116" t="s">
-        <v>1763</v>
+        <v>1762</v>
       </c>
       <c r="L50" s="116" t="str">
         <f aca="false">IF(D50&lt;&gt;"","Suggested by "&amp;IF(Partner_Name="","your provider",Partner_Name),G50)</f>
@@ -32961,26 +32959,26 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="1" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="C51" s="109" t="n">
         <v>0.01</v>
       </c>
       <c r="D51" s="109"/>
       <c r="G51" s="107" t="s">
+        <v>1764</v>
+      </c>
+      <c r="H51" s="116" t="s">
         <v>1765</v>
-      </c>
-      <c r="H51" s="116" t="s">
-        <v>1766</v>
       </c>
       <c r="I51" s="116" t="s">
         <v>1621</v>
       </c>
       <c r="J51" s="116" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="K51" s="116" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="L51" s="116" t="str">
         <f aca="false">IF(D51&lt;&gt;"","Suggested by "&amp;IF(Partner_Name="","your provider",Partner_Name),G51)</f>
@@ -32993,82 +32991,82 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="115" t="s">
-        <v>1768</v>
+        <v>1767</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="1" t="s">
-        <v>1769</v>
+        <v>1768</v>
       </c>
       <c r="C53" s="107" t="n">
         <v>83</v>
       </c>
       <c r="G53" s="107" t="s">
+        <v>1769</v>
+      </c>
+      <c r="H53" s="116" t="s">
         <v>1770</v>
       </c>
-      <c r="H53" s="116" t="s">
+      <c r="I53" s="116" t="s">
         <v>1771</v>
-      </c>
-      <c r="I53" s="116" t="s">
-        <v>1772</v>
       </c>
       <c r="J53" s="116"/>
       <c r="K53" s="116" t="s">
-        <v>1773</v>
+        <v>1772</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="1" t="s">
-        <v>1774</v>
+        <v>1773</v>
       </c>
       <c r="C54" s="107" t="n">
         <v>86</v>
       </c>
       <c r="G54" s="107" t="s">
+        <v>1769</v>
+      </c>
+      <c r="H54" s="116" t="s">
         <v>1770</v>
       </c>
-      <c r="H54" s="116" t="s">
-        <v>1771</v>
-      </c>
       <c r="I54" s="116" t="s">
-        <v>1775</v>
+        <v>1774</v>
       </c>
       <c r="J54" s="116"/>
       <c r="K54" s="116" t="s">
-        <v>1773</v>
+        <v>1772</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="115" t="s">
-        <v>1776</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="1" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="C56" s="121" t="n">
         <v>0.039</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="1" t="s">
-        <v>1779</v>
+        <v>1778</v>
       </c>
       <c r="C57" s="122" t="n">
         <v>0.23</v>
       </c>
       <c r="G57" s="1" t="s">
+        <v>1779</v>
+      </c>
+      <c r="H57" s="1" t="s">
         <v>1780</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="I57" s="1" t="s">
         <v>1781</v>
-      </c>
-      <c r="I57" s="1" t="s">
-        <v>1782</v>
       </c>
     </row>
   </sheetData>
@@ -33105,17 +33103,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="20" t="s">
-        <v>1783</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="123" t="s">
-        <v>1784</v>
+        <v>1783</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="124" t="s">
-        <v>1785</v>
+        <v>1784</v>
       </c>
       <c r="C3" s="124"/>
       <c r="D3" s="124"/>
@@ -33125,7 +33123,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
-        <v>1786</v>
+        <v>1785</v>
       </c>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
@@ -33136,40 +33134,40 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C6" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="D6" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="E6" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="F6" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="G6" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="H6" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
-        <v>1794</v>
+        <v>1793</v>
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15"/>
       <c r="E7" s="125" t="s">
-        <v>1795</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="13" t="s">
-        <v>1796</v>
+        <v>1795</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14"/>
@@ -33180,352 +33178,352 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C9" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="D9" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="E9" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="F9" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="G9" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="H9" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="25" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="C10" s="126" t="n">
         <v>44000</v>
       </c>
       <c r="D10" s="17" t="s">
+        <v>1797</v>
+      </c>
+      <c r="E10" s="125" t="s">
         <v>1798</v>
       </c>
-      <c r="E10" s="125" t="s">
+      <c r="F10" s="17" t="s">
         <v>1799</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="G10" s="127" t="s">
         <v>1800</v>
       </c>
-      <c r="G10" s="127" t="s">
+      <c r="H10" s="125" t="s">
         <v>1801</v>
-      </c>
-      <c r="H10" s="125" t="s">
-        <v>1802</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="25" t="s">
-        <v>1803</v>
+        <v>1802</v>
       </c>
       <c r="C11" s="126" t="n">
         <v>48000</v>
       </c>
       <c r="D11" s="17" t="s">
+        <v>1803</v>
+      </c>
+      <c r="E11" s="125" t="s">
         <v>1804</v>
       </c>
-      <c r="E11" s="125" t="s">
+      <c r="F11" s="17" t="s">
+        <v>1799</v>
+      </c>
+      <c r="G11" s="127" t="s">
         <v>1805</v>
       </c>
-      <c r="F11" s="17" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G11" s="127" t="s">
+      <c r="H11" s="125" t="s">
         <v>1806</v>
-      </c>
-      <c r="H11" s="125" t="s">
-        <v>1807</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="25" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
       <c r="C12" s="126" t="n">
         <v>53000</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E12" s="125" t="s">
+        <v>1798</v>
+      </c>
+      <c r="F12" s="17" t="s">
         <v>1799</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="G12" s="127" t="s">
         <v>1800</v>
       </c>
-      <c r="G12" s="127" t="s">
-        <v>1801</v>
-      </c>
       <c r="H12" s="125" t="s">
-        <v>1809</v>
+        <v>1808</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="25" t="s">
-        <v>1810</v>
+        <v>1809</v>
       </c>
       <c r="C13" s="126" t="n">
         <v>35000</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E13" s="125" t="s">
+        <v>1798</v>
+      </c>
+      <c r="F13" s="17" t="s">
         <v>1799</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="G13" s="127" t="s">
         <v>1800</v>
       </c>
-      <c r="G13" s="127" t="s">
-        <v>1801</v>
-      </c>
       <c r="H13" s="125" t="s">
-        <v>1811</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="25" t="s">
-        <v>1812</v>
+        <v>1811</v>
       </c>
       <c r="C14" s="128" t="n">
         <v>0.2</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E14" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G14" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H14" s="125" t="s">
-        <v>1813</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="25" t="s">
-        <v>1814</v>
+        <v>1813</v>
       </c>
       <c r="C15" s="128" t="n">
         <v>0.4</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>1815</v>
+        <v>1814</v>
       </c>
       <c r="E15" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G15" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H15" s="125" t="s">
-        <v>1813</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="25" t="s">
-        <v>1816</v>
+        <v>1815</v>
       </c>
       <c r="C16" s="126" t="n">
         <v>2000</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E16" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G16" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H16" s="125" t="s">
-        <v>1817</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="25" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
       <c r="C17" s="126" t="n">
         <v>4000</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E17" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="F17" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G17" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H17" s="125" t="s">
-        <v>1817</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="25" t="s">
-        <v>1819</v>
+        <v>1818</v>
       </c>
       <c r="C18" s="126" t="n">
         <v>2000</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E18" s="125" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F18" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G18" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H18" s="125" t="s">
-        <v>1821</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="25" t="s">
-        <v>1822</v>
+        <v>1821</v>
       </c>
       <c r="C19" s="128" t="n">
         <v>0.2</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E19" s="125" t="s">
-        <v>1823</v>
+        <v>1822</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G19" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H19" s="125" t="s">
-        <v>1821</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="25" t="s">
-        <v>1824</v>
+        <v>1823</v>
       </c>
       <c r="C20" s="126" t="n">
         <v>1900</v>
       </c>
       <c r="D20" s="17" t="s">
+        <v>1803</v>
+      </c>
+      <c r="E20" s="125" t="s">
         <v>1804</v>
       </c>
-      <c r="E20" s="125" t="s">
+      <c r="F20" s="17" t="s">
+        <v>1799</v>
+      </c>
+      <c r="G20" s="127" t="s">
         <v>1805</v>
       </c>
-      <c r="F20" s="17" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G20" s="127" t="s">
+      <c r="H20" s="125" t="s">
         <v>1806</v>
-      </c>
-      <c r="H20" s="125" t="s">
-        <v>1807</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="25" t="s">
-        <v>1825</v>
+        <v>1824</v>
       </c>
       <c r="C21" s="126" t="n">
         <v>1000</v>
       </c>
       <c r="D21" s="17" t="s">
+        <v>1803</v>
+      </c>
+      <c r="E21" s="125" t="s">
         <v>1804</v>
       </c>
-      <c r="E21" s="125" t="s">
+      <c r="F21" s="17" t="s">
+        <v>1825</v>
+      </c>
+      <c r="G21" s="127" t="s">
         <v>1805</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="H21" s="125" t="s">
         <v>1826</v>
-      </c>
-      <c r="G21" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H21" s="125" t="s">
-        <v>1827</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="25" t="s">
-        <v>1828</v>
+        <v>1827</v>
       </c>
       <c r="C22" s="126" t="n">
         <v>2000</v>
       </c>
       <c r="D22" s="17" t="s">
+        <v>1803</v>
+      </c>
+      <c r="E22" s="125" t="s">
         <v>1804</v>
       </c>
-      <c r="E22" s="125" t="s">
+      <c r="F22" s="17" t="s">
+        <v>1825</v>
+      </c>
+      <c r="G22" s="127" t="s">
         <v>1805</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="H22" s="125" t="s">
         <v>1826</v>
-      </c>
-      <c r="G22" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H22" s="125" t="s">
-        <v>1827</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="25" t="s">
-        <v>1829</v>
+        <v>1828</v>
       </c>
       <c r="C23" s="126" t="n">
         <v>1950</v>
       </c>
       <c r="D23" s="17" t="s">
+        <v>1803</v>
+      </c>
+      <c r="E23" s="125" t="s">
         <v>1804</v>
-      </c>
-      <c r="E23" s="125" t="s">
-        <v>1805</v>
       </c>
       <c r="F23" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G23" s="127" t="s">
+        <v>1829</v>
+      </c>
+      <c r="H23" s="125" t="s">
         <v>1830</v>
-      </c>
-      <c r="H23" s="125" t="s">
-        <v>1831</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="13" t="s">
-        <v>1832</v>
+        <v>1831</v>
       </c>
       <c r="C24" s="14"/>
       <c r="D24" s="14"/>
@@ -33536,224 +33534,224 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C25" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="D25" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D25" s="16" t="s">
+      <c r="E25" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E25" s="16" t="s">
+      <c r="F25" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F25" s="16" t="s">
+      <c r="G25" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G25" s="16" t="s">
+      <c r="H25" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H25" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="25" t="s">
-        <v>1833</v>
+        <v>1832</v>
       </c>
       <c r="C26" s="126" t="n">
         <v>13000</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E26" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="F26" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G26" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H26" s="125" t="s">
-        <v>1834</v>
+        <v>1833</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="25" t="s">
-        <v>1835</v>
+        <v>1834</v>
       </c>
       <c r="C27" s="126" t="n">
         <v>12012</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E27" s="125" t="s">
+        <v>1798</v>
+      </c>
+      <c r="F27" s="17" t="s">
         <v>1799</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="G27" s="127" t="s">
         <v>1800</v>
       </c>
-      <c r="G27" s="127" t="s">
-        <v>1801</v>
-      </c>
       <c r="H27" s="125" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="25" t="s">
-        <v>1837</v>
+        <v>1836</v>
       </c>
       <c r="C28" s="126" t="n">
         <v>28700</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E28" s="125" t="s">
+        <v>1798</v>
+      </c>
+      <c r="F28" s="17" t="s">
         <v>1799</v>
       </c>
-      <c r="F28" s="17" t="s">
+      <c r="G28" s="127" t="s">
         <v>1800</v>
       </c>
-      <c r="G28" s="127" t="s">
-        <v>1801</v>
-      </c>
       <c r="H28" s="125" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="25" t="s">
-        <v>1838</v>
+        <v>1837</v>
       </c>
       <c r="C29" s="126" t="n">
         <v>70044</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E29" s="125" t="s">
+        <v>1798</v>
+      </c>
+      <c r="F29" s="17" t="s">
         <v>1799</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="G29" s="127" t="s">
         <v>1800</v>
       </c>
-      <c r="G29" s="127" t="s">
-        <v>1801</v>
-      </c>
       <c r="H29" s="125" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="25" t="s">
-        <v>1839</v>
+        <v>1838</v>
       </c>
       <c r="C30" s="129" t="n">
         <v>0.005</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E30" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="F30" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G30" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H30" s="125" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="25" t="s">
-        <v>1840</v>
+        <v>1839</v>
       </c>
       <c r="C31" s="129" t="n">
         <v>0.02</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E31" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="F31" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G31" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H31" s="125" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="25" t="s">
-        <v>1841</v>
+        <v>1840</v>
       </c>
       <c r="C32" s="129" t="n">
         <v>0.03</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E32" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="F32" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G32" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H32" s="125" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="25" t="s">
-        <v>1842</v>
+        <v>1841</v>
       </c>
       <c r="C33" s="129" t="n">
         <v>0.08</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E33" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="F33" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G33" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H33" s="125" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="15" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="C34" s="15"/>
       <c r="D34" s="15"/>
       <c r="E34" s="125" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="13" t="s">
-        <v>1844</v>
+        <v>1843</v>
       </c>
       <c r="C35" s="14"/>
       <c r="D35" s="14"/>
@@ -33764,178 +33762,178 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C36" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="D36" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D36" s="16" t="s">
+      <c r="E36" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E36" s="16" t="s">
+      <c r="F36" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F36" s="16" t="s">
+      <c r="G36" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G36" s="16" t="s">
+      <c r="H36" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H36" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="25" t="s">
-        <v>1845</v>
+        <v>1844</v>
       </c>
       <c r="C37" s="130" t="n">
         <v>0.0435</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E37" s="125" t="s">
+        <v>1845</v>
+      </c>
+      <c r="F37" s="17" t="s">
         <v>1846</v>
       </c>
-      <c r="F37" s="17" t="s">
+      <c r="G37" s="127" t="s">
+        <v>1800</v>
+      </c>
+      <c r="H37" s="125" t="s">
         <v>1847</v>
-      </c>
-      <c r="G37" s="127" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H37" s="125" t="s">
-        <v>1848</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="25" t="s">
-        <v>1849</v>
+        <v>1848</v>
       </c>
       <c r="C38" s="131" t="n">
         <v>0.042375</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>1850</v>
+        <v>1849</v>
       </c>
       <c r="E38" s="125" t="s">
-        <v>1846</v>
+        <v>1845</v>
       </c>
       <c r="F38" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G38" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H38" s="125" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="25" t="s">
-        <v>1852</v>
+        <v>1851</v>
       </c>
       <c r="C39" s="126" t="n">
         <v>352</v>
       </c>
       <c r="D39" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E39" s="125" t="s">
-        <v>1853</v>
+        <v>1852</v>
       </c>
       <c r="F39" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G39" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H39" s="125" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="25" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
       <c r="C40" s="126" t="n">
         <v>12</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E40" s="125" t="s">
-        <v>1823</v>
+        <v>1822</v>
       </c>
       <c r="F40" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G40" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H40" s="125" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="25" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
       <c r="C41" s="126" t="n">
         <v>424</v>
       </c>
       <c r="D41" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E41" s="125" t="s">
-        <v>1823</v>
+        <v>1822</v>
       </c>
       <c r="F41" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G41" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H41" s="125" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="25" t="s">
-        <v>1857</v>
+        <v>1856</v>
       </c>
       <c r="C42" s="132" t="n">
         <v>6</v>
       </c>
       <c r="D42" s="17" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E42" s="125" t="s">
-        <v>1823</v>
+        <v>1822</v>
       </c>
       <c r="F42" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G42" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H42" s="125" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="15" t="s">
-        <v>1858</v>
+        <v>1857</v>
       </c>
       <c r="C43" s="15"/>
       <c r="D43" s="15"/>
       <c r="E43" s="125" t="s">
-        <v>1859</v>
+        <v>1858</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="13" t="s">
-        <v>1860</v>
+        <v>1859</v>
       </c>
       <c r="C44" s="14"/>
       <c r="D44" s="14"/>
@@ -33946,30 +33944,30 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="D45" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D45" s="16" t="s">
+      <c r="E45" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E45" s="16" t="s">
+      <c r="F45" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F45" s="16" t="s">
+      <c r="G45" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G45" s="16" t="s">
+      <c r="H45" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H45" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="25" t="s">
-        <v>1861</v>
+        <v>1860</v>
       </c>
       <c r="C46" s="133" t="n">
         <v>0</v>
@@ -33978,21 +33976,21 @@
         <v>0.15</v>
       </c>
       <c r="E46" s="134" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F46" s="12" t="s">
         <v>1862</v>
       </c>
-      <c r="F46" s="12" t="s">
+      <c r="G46" s="135" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H46" s="134" t="s">
         <v>1863</v>
-      </c>
-      <c r="G46" s="135" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H46" s="134" t="s">
-        <v>1864</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="25" t="s">
-        <v>1865</v>
+        <v>1864</v>
       </c>
       <c r="C47" s="133" t="n">
         <v>30</v>
@@ -34001,21 +33999,21 @@
         <v>0.2</v>
       </c>
       <c r="E47" s="134" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F47" s="12" t="s">
         <v>1862</v>
       </c>
-      <c r="F47" s="12" t="s">
+      <c r="G47" s="135" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H47" s="134" t="s">
         <v>1863</v>
-      </c>
-      <c r="G47" s="135" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H47" s="134" t="s">
-        <v>1864</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="25" t="s">
-        <v>1866</v>
+        <v>1865</v>
       </c>
       <c r="C48" s="133" t="n">
         <v>40</v>
@@ -34024,21 +34022,21 @@
         <v>0.25</v>
       </c>
       <c r="E48" s="134" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F48" s="12" t="s">
         <v>1862</v>
       </c>
-      <c r="F48" s="12" t="s">
+      <c r="G48" s="135" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H48" s="134" t="s">
         <v>1863</v>
-      </c>
-      <c r="G48" s="135" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H48" s="134" t="s">
-        <v>1864</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="25" t="s">
-        <v>1867</v>
+        <v>1866</v>
       </c>
       <c r="C49" s="133" t="n">
         <v>50</v>
@@ -34047,21 +34045,21 @@
         <v>0.3</v>
       </c>
       <c r="E49" s="134" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F49" s="12" t="s">
         <v>1862</v>
       </c>
-      <c r="F49" s="12" t="s">
+      <c r="G49" s="135" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H49" s="134" t="s">
         <v>1863</v>
-      </c>
-      <c r="G49" s="135" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H49" s="134" t="s">
-        <v>1864</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="25" t="s">
-        <v>1868</v>
+        <v>1867</v>
       </c>
       <c r="C50" s="133" t="n">
         <v>55</v>
@@ -34070,21 +34068,21 @@
         <v>0.35</v>
       </c>
       <c r="E50" s="134" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F50" s="12" t="s">
         <v>1862</v>
       </c>
-      <c r="F50" s="12" t="s">
+      <c r="G50" s="135" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H50" s="134" t="s">
         <v>1863</v>
-      </c>
-      <c r="G50" s="135" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H50" s="134" t="s">
-        <v>1864</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="25" t="s">
-        <v>1869</v>
+        <v>1868</v>
       </c>
       <c r="C51" s="133" t="n">
         <v>60</v>
@@ -34093,21 +34091,21 @@
         <v>0.4</v>
       </c>
       <c r="E51" s="134" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F51" s="12" t="s">
         <v>1862</v>
       </c>
-      <c r="F51" s="12" t="s">
+      <c r="G51" s="135" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H51" s="134" t="s">
         <v>1863</v>
-      </c>
-      <c r="G51" s="135" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H51" s="134" t="s">
-        <v>1864</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="25" t="s">
-        <v>1870</v>
+        <v>1869</v>
       </c>
       <c r="C52" s="126" t="n">
         <v>115000</v>
@@ -34116,21 +34114,21 @@
         <v>138</v>
       </c>
       <c r="E52" s="125" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F52" s="17" t="s">
         <v>1862</v>
       </c>
-      <c r="F52" s="17" t="s">
-        <v>1863</v>
-      </c>
       <c r="G52" s="127" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="H52" s="125" t="s">
-        <v>1871</v>
+        <v>1870</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="25" t="s">
-        <v>1872</v>
+        <v>1871</v>
       </c>
       <c r="C53" s="128" t="n">
         <v>0.25</v>
@@ -34139,21 +34137,21 @@
         <v>58</v>
       </c>
       <c r="E53" s="125" t="s">
+        <v>1872</v>
+      </c>
+      <c r="F53" s="17" t="s">
         <v>1873</v>
       </c>
-      <c r="F53" s="17" t="s">
+      <c r="G53" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H53" s="125" t="s">
         <v>1874</v>
-      </c>
-      <c r="G53" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H53" s="125" t="s">
-        <v>1875</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="25" t="s">
-        <v>1876</v>
+        <v>1875</v>
       </c>
       <c r="C54" s="126" t="n">
         <v>200000</v>
@@ -34162,21 +34160,21 @@
         <v>58</v>
       </c>
       <c r="E54" s="125" t="s">
+        <v>1872</v>
+      </c>
+      <c r="F54" s="17" t="s">
         <v>1873</v>
       </c>
-      <c r="F54" s="17" t="s">
+      <c r="G54" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H54" s="125" t="s">
         <v>1874</v>
-      </c>
-      <c r="G54" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H54" s="125" t="s">
-        <v>1875</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="25" t="s">
-        <v>1877</v>
+        <v>1876</v>
       </c>
       <c r="C55" s="126" t="n">
         <v>500000</v>
@@ -34185,21 +34183,21 @@
         <v>58</v>
       </c>
       <c r="E55" s="125" t="s">
+        <v>1872</v>
+      </c>
+      <c r="F55" s="17" t="s">
         <v>1873</v>
       </c>
-      <c r="F55" s="17" t="s">
+      <c r="G55" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H55" s="125" t="s">
         <v>1874</v>
-      </c>
-      <c r="G55" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H55" s="125" t="s">
-        <v>1875</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="25" t="s">
-        <v>1878</v>
+        <v>1877</v>
       </c>
       <c r="C56" s="128" t="n">
         <v>0.2</v>
@@ -34208,100 +34206,100 @@
         <v>58</v>
       </c>
       <c r="E56" s="125" t="s">
+        <v>1872</v>
+      </c>
+      <c r="F56" s="17" t="s">
         <v>1873</v>
       </c>
-      <c r="F56" s="17" t="s">
+      <c r="G56" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H56" s="125" t="s">
         <v>1874</v>
-      </c>
-      <c r="G56" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H56" s="125" t="s">
-        <v>1875</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="25" t="s">
-        <v>1879</v>
+        <v>1878</v>
       </c>
       <c r="C57" s="126" t="n">
         <v>2200000</v>
       </c>
       <c r="D57" s="17" t="s">
+        <v>1879</v>
+      </c>
+      <c r="E57" s="125" t="s">
+        <v>1872</v>
+      </c>
+      <c r="F57" s="17" t="s">
+        <v>1799</v>
+      </c>
+      <c r="G57" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H57" s="125" t="s">
         <v>1880</v>
-      </c>
-      <c r="E57" s="125" t="s">
-        <v>1873</v>
-      </c>
-      <c r="F57" s="17" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G57" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H57" s="125" t="s">
-        <v>1881</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="25" t="s">
-        <v>1882</v>
+        <v>1881</v>
       </c>
       <c r="C58" s="128" t="n">
         <v>0.4</v>
       </c>
       <c r="D58" s="17" t="s">
+        <v>1879</v>
+      </c>
+      <c r="E58" s="125" t="s">
+        <v>1872</v>
+      </c>
+      <c r="F58" s="17" t="s">
+        <v>1882</v>
+      </c>
+      <c r="G58" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H58" s="125" t="s">
         <v>1880</v>
-      </c>
-      <c r="E58" s="125" t="s">
-        <v>1873</v>
-      </c>
-      <c r="F58" s="17" t="s">
-        <v>1883</v>
-      </c>
-      <c r="G58" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H58" s="125" t="s">
-        <v>1881</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="25" t="s">
-        <v>1884</v>
+        <v>1883</v>
       </c>
       <c r="C59" s="132" t="n">
         <v>60</v>
       </c>
       <c r="D59" s="17" t="s">
-        <v>1880</v>
+        <v>1879</v>
       </c>
       <c r="E59" s="125" t="s">
+        <v>1884</v>
+      </c>
+      <c r="F59" s="17" t="s">
+        <v>1882</v>
+      </c>
+      <c r="G59" s="127" t="s">
         <v>1885</v>
       </c>
-      <c r="F59" s="17" t="s">
-        <v>1883</v>
-      </c>
-      <c r="G59" s="127" t="s">
+      <c r="H59" s="125" t="s">
         <v>1886</v>
-      </c>
-      <c r="H59" s="125" t="s">
-        <v>1887</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="15" t="s">
-        <v>1888</v>
+        <v>1887</v>
       </c>
       <c r="C60" s="15"/>
       <c r="D60" s="15"/>
       <c r="E60" s="125" t="s">
-        <v>1889</v>
+        <v>1888</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="13" t="s">
-        <v>1890</v>
+        <v>1889</v>
       </c>
       <c r="C61" s="14"/>
       <c r="D61" s="14"/>
@@ -34312,100 +34310,100 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C62" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C62" s="16" t="s">
+      <c r="D62" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D62" s="16" t="s">
+      <c r="E62" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E62" s="16" t="s">
+      <c r="F62" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F62" s="16" t="s">
+      <c r="G62" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G62" s="16" t="s">
+      <c r="H62" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H62" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="25" t="s">
-        <v>1891</v>
+        <v>1890</v>
       </c>
       <c r="C63" s="136" t="n">
         <v>299.3</v>
       </c>
       <c r="D63" s="17" t="s">
+        <v>1891</v>
+      </c>
+      <c r="E63" s="125" t="s">
         <v>1892</v>
       </c>
-      <c r="E63" s="125" t="s">
+      <c r="F63" s="17" t="s">
+        <v>1799</v>
+      </c>
+      <c r="G63" s="127" t="s">
+        <v>1800</v>
+      </c>
+      <c r="H63" s="125" t="s">
         <v>1893</v>
-      </c>
-      <c r="F63" s="17" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G63" s="127" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H63" s="125" t="s">
-        <v>1894</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="25" t="s">
-        <v>1895</v>
+        <v>1894</v>
       </c>
       <c r="C64" s="136" t="n">
         <f aca="false">State_Pension_Week*Weeks_Per_Year</f>
         <v>15563.6</v>
       </c>
       <c r="D64" s="17" t="s">
-        <v>1896</v>
+        <v>1895</v>
       </c>
       <c r="E64" s="125" t="s">
+        <v>1892</v>
+      </c>
+      <c r="F64" s="17" t="s">
+        <v>1799</v>
+      </c>
+      <c r="G64" s="127" t="s">
+        <v>1800</v>
+      </c>
+      <c r="H64" s="125" t="s">
         <v>1893</v>
-      </c>
-      <c r="F64" s="17" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G64" s="127" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H64" s="125" t="s">
-        <v>1894</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="25" t="s">
-        <v>1897</v>
+        <v>1896</v>
       </c>
       <c r="C65" s="132" t="n">
         <v>66</v>
       </c>
       <c r="D65" s="17" t="s">
+        <v>1897</v>
+      </c>
+      <c r="E65" s="125" t="s">
         <v>1898</v>
       </c>
-      <c r="E65" s="125" t="s">
+      <c r="F65" s="17" t="s">
+        <v>1882</v>
+      </c>
+      <c r="G65" s="127" t="s">
+        <v>1800</v>
+      </c>
+      <c r="H65" s="125" t="s">
         <v>1899</v>
-      </c>
-      <c r="F65" s="17" t="s">
-        <v>1883</v>
-      </c>
-      <c r="G65" s="127" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H65" s="125" t="s">
-        <v>1900</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="25" t="s">
-        <v>1901</v>
+        <v>1900</v>
       </c>
       <c r="C66" s="136" t="n">
         <v>259.5</v>
@@ -34414,44 +34412,44 @@
         <v>77</v>
       </c>
       <c r="E66" s="125" t="s">
+        <v>1901</v>
+      </c>
+      <c r="F66" s="17" t="s">
+        <v>1799</v>
+      </c>
+      <c r="G66" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H66" s="125" t="s">
         <v>1902</v>
-      </c>
-      <c r="F66" s="17" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G66" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H66" s="125" t="s">
-        <v>1903</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="25" t="s">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="C67" s="136" t="n">
         <v>299.3</v>
       </c>
       <c r="D67" s="17" t="s">
-        <v>1905</v>
+        <v>1904</v>
       </c>
       <c r="E67" s="125" t="s">
-        <v>1823</v>
+        <v>1822</v>
       </c>
       <c r="F67" s="17" t="s">
-        <v>1800</v>
+        <v>1799</v>
       </c>
       <c r="G67" s="127" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="H67" s="125" t="s">
-        <v>1903</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="25" t="s">
-        <v>1906</v>
+        <v>1905</v>
       </c>
       <c r="C68" s="136" t="n">
         <v>254</v>
@@ -34460,21 +34458,21 @@
         <v>80</v>
       </c>
       <c r="E68" s="125" t="s">
+        <v>1906</v>
+      </c>
+      <c r="F68" s="17" t="s">
+        <v>1799</v>
+      </c>
+      <c r="G68" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H68" s="125" t="s">
         <v>1907</v>
-      </c>
-      <c r="F68" s="17" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G68" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H68" s="125" t="s">
-        <v>1908</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="25" t="s">
-        <v>1909</v>
+        <v>1908</v>
       </c>
       <c r="C69" s="128" t="n">
         <v>0.75</v>
@@ -34483,44 +34481,44 @@
         <v>80</v>
       </c>
       <c r="E69" s="125" t="s">
+        <v>1909</v>
+      </c>
+      <c r="F69" s="17" t="s">
         <v>1910</v>
       </c>
-      <c r="F69" s="17" t="s">
+      <c r="G69" s="127" t="s">
         <v>1911</v>
       </c>
-      <c r="G69" s="127" t="s">
+      <c r="H69" s="125" t="s">
         <v>1912</v>
-      </c>
-      <c r="H69" s="125" t="s">
-        <v>1913</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B70" s="25" t="s">
-        <v>1914</v>
+        <v>1913</v>
       </c>
       <c r="C70" s="132" t="n">
         <v>52</v>
       </c>
       <c r="D70" s="17" t="s">
+        <v>1914</v>
+      </c>
+      <c r="E70" s="125" t="s">
         <v>1915</v>
       </c>
-      <c r="E70" s="125" t="s">
-        <v>1916</v>
-      </c>
       <c r="F70" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G70" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H70" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B71" s="13" t="s">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="C71" s="14"/>
       <c r="D71" s="14"/>
@@ -34531,122 +34529,122 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C72" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C72" s="16" t="s">
+      <c r="D72" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D72" s="16" t="s">
+      <c r="E72" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E72" s="16" t="s">
+      <c r="F72" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F72" s="16" t="s">
+      <c r="G72" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G72" s="16" t="s">
+      <c r="H72" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H72" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B73" s="25" t="s">
-        <v>1918</v>
+        <v>1917</v>
       </c>
       <c r="C73" s="128" t="n">
         <v>0.33</v>
       </c>
       <c r="D73" s="17" t="s">
+        <v>1918</v>
+      </c>
+      <c r="E73" s="125" t="s">
         <v>1919</v>
-      </c>
-      <c r="E73" s="125" t="s">
-        <v>1920</v>
       </c>
       <c r="F73" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G73" s="127" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="H73" s="125" t="s">
-        <v>1921</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B74" s="25" t="s">
-        <v>1922</v>
+        <v>1921</v>
       </c>
       <c r="C74" s="128" t="n">
         <v>0.38</v>
       </c>
       <c r="D74" s="17" t="s">
-        <v>1919</v>
+        <v>1918</v>
       </c>
       <c r="E74" s="125" t="s">
+        <v>1922</v>
+      </c>
+      <c r="F74" s="17" t="s">
+        <v>1799</v>
+      </c>
+      <c r="G74" s="127" t="s">
+        <v>1800</v>
+      </c>
+      <c r="H74" s="125" t="s">
         <v>1923</v>
-      </c>
-      <c r="F74" s="17" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G74" s="127" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H74" s="125" t="s">
-        <v>1924</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="25" t="s">
-        <v>1925</v>
+        <v>1924</v>
       </c>
       <c r="C75" s="132" t="n">
         <v>8</v>
       </c>
       <c r="D75" s="17" t="s">
+        <v>1925</v>
+      </c>
+      <c r="E75" s="125" t="s">
         <v>1926</v>
-      </c>
-      <c r="E75" s="125" t="s">
-        <v>1927</v>
       </c>
       <c r="F75" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G75" s="127" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="H75" s="125" t="s">
-        <v>1928</v>
+        <v>1927</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="25" t="s">
-        <v>1929</v>
+        <v>1928</v>
       </c>
       <c r="C76" s="128" t="n">
         <v>0.01</v>
       </c>
       <c r="D76" s="17" t="s">
+        <v>1929</v>
+      </c>
+      <c r="E76" s="125" t="s">
         <v>1930</v>
-      </c>
-      <c r="E76" s="125" t="s">
-        <v>1931</v>
       </c>
       <c r="F76" s="17" t="s">
         <v>1621</v>
       </c>
       <c r="G76" s="127" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="H76" s="125" t="s">
-        <v>1932</v>
+        <v>1931</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="13" t="s">
-        <v>1933</v>
+        <v>1932</v>
       </c>
       <c r="C77" s="14"/>
       <c r="D77" s="14"/>
@@ -34657,30 +34655,30 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B78" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C78" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C78" s="16" t="s">
+      <c r="D78" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D78" s="16" t="s">
+      <c r="E78" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E78" s="16" t="s">
+      <c r="F78" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F78" s="16" t="s">
+      <c r="G78" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G78" s="16" t="s">
+      <c r="H78" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H78" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B79" s="25" t="s">
-        <v>1934</v>
+        <v>1933</v>
       </c>
       <c r="C79" s="137" t="n">
         <v>4</v>
@@ -34689,21 +34687,21 @@
         <v>33</v>
       </c>
       <c r="E79" s="125" t="s">
+        <v>1934</v>
+      </c>
+      <c r="F79" s="17" t="s">
         <v>1935</v>
       </c>
-      <c r="F79" s="17" t="s">
+      <c r="G79" s="127" t="s">
+        <v>1800</v>
+      </c>
+      <c r="H79" s="125" t="s">
         <v>1936</v>
-      </c>
-      <c r="G79" s="127" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H79" s="125" t="s">
-        <v>1937</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B80" s="25" t="s">
-        <v>1938</v>
+        <v>1937</v>
       </c>
       <c r="C80" s="137" t="n">
         <v>3.5</v>
@@ -34712,203 +34710,203 @@
         <v>33</v>
       </c>
       <c r="E80" s="125" t="s">
+        <v>1934</v>
+      </c>
+      <c r="F80" s="17" t="s">
         <v>1935</v>
       </c>
-      <c r="F80" s="17" t="s">
+      <c r="G80" s="127" t="s">
+        <v>1800</v>
+      </c>
+      <c r="H80" s="125" t="s">
         <v>1936</v>
-      </c>
-      <c r="G80" s="127" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H80" s="125" t="s">
-        <v>1937</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B81" s="25" t="s">
-        <v>1939</v>
+        <v>1938</v>
       </c>
       <c r="C81" s="128" t="n">
         <v>0.9</v>
       </c>
       <c r="D81" s="17" t="s">
+        <v>1939</v>
+      </c>
+      <c r="E81" s="125" t="s">
+        <v>1934</v>
+      </c>
+      <c r="F81" s="17" t="s">
+        <v>1935</v>
+      </c>
+      <c r="G81" s="127" t="s">
+        <v>1800</v>
+      </c>
+      <c r="H81" s="125" t="s">
         <v>1940</v>
-      </c>
-      <c r="E81" s="125" t="s">
-        <v>1935</v>
-      </c>
-      <c r="F81" s="17" t="s">
-        <v>1936</v>
-      </c>
-      <c r="G81" s="127" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H81" s="125" t="s">
-        <v>1941</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B82" s="25" t="s">
-        <v>1942</v>
+        <v>1941</v>
       </c>
       <c r="C82" s="128" t="n">
         <f aca="false">1-LTV_Max</f>
         <v>0.1</v>
       </c>
       <c r="D82" s="17" t="s">
+        <v>1942</v>
+      </c>
+      <c r="E82" s="125" t="s">
         <v>1943</v>
       </c>
-      <c r="E82" s="125" t="s">
+      <c r="F82" s="17" t="s">
+        <v>1935</v>
+      </c>
+      <c r="G82" s="127" t="s">
+        <v>1800</v>
+      </c>
+      <c r="H82" s="125" t="s">
         <v>1944</v>
-      </c>
-      <c r="F82" s="17" t="s">
-        <v>1936</v>
-      </c>
-      <c r="G82" s="127" t="s">
-        <v>1801</v>
-      </c>
-      <c r="H82" s="125" t="s">
-        <v>1945</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B83" s="15" t="s">
-        <v>1946</v>
+        <v>1945</v>
       </c>
       <c r="C83" s="15"/>
       <c r="D83" s="15"/>
       <c r="E83" s="125" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B84" s="25" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="C84" s="128" t="n">
         <v>0.01</v>
       </c>
       <c r="D84" s="17" t="s">
+        <v>1948</v>
+      </c>
+      <c r="E84" s="125" t="s">
         <v>1949</v>
       </c>
-      <c r="E84" s="125" t="s">
+      <c r="F84" s="17" t="s">
         <v>1950</v>
       </c>
-      <c r="F84" s="17" t="s">
+      <c r="G84" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H84" s="125" t="s">
         <v>1951</v>
-      </c>
-      <c r="G84" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H84" s="125" t="s">
-        <v>1952</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B85" s="25" t="s">
-        <v>1953</v>
+        <v>1952</v>
       </c>
       <c r="C85" s="126" t="n">
         <v>1000000</v>
       </c>
       <c r="D85" s="17" t="s">
+        <v>1948</v>
+      </c>
+      <c r="E85" s="125" t="s">
         <v>1949</v>
       </c>
-      <c r="E85" s="125" t="s">
+      <c r="F85" s="17" t="s">
         <v>1950</v>
       </c>
-      <c r="F85" s="17" t="s">
+      <c r="G85" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H85" s="125" t="s">
         <v>1951</v>
-      </c>
-      <c r="G85" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H85" s="125" t="s">
-        <v>1952</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B86" s="25" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="C86" s="128" t="n">
         <v>0.02</v>
       </c>
       <c r="D86" s="17" t="s">
+        <v>1948</v>
+      </c>
+      <c r="E86" s="125" t="s">
         <v>1949</v>
       </c>
-      <c r="E86" s="125" t="s">
+      <c r="F86" s="17" t="s">
         <v>1950</v>
       </c>
-      <c r="F86" s="17" t="s">
+      <c r="G86" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H86" s="125" t="s">
         <v>1951</v>
-      </c>
-      <c r="G86" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H86" s="125" t="s">
-        <v>1952</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B87" s="25" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="C87" s="126" t="n">
         <v>1500000</v>
       </c>
       <c r="D87" s="17" t="s">
+        <v>1948</v>
+      </c>
+      <c r="E87" s="125" t="s">
         <v>1949</v>
       </c>
-      <c r="E87" s="125" t="s">
+      <c r="F87" s="17" t="s">
         <v>1950</v>
       </c>
-      <c r="F87" s="17" t="s">
+      <c r="G87" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H87" s="125" t="s">
         <v>1951</v>
-      </c>
-      <c r="G87" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H87" s="125" t="s">
-        <v>1952</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="25" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
       <c r="C88" s="128" t="n">
         <v>0.06</v>
       </c>
       <c r="D88" s="17" t="s">
+        <v>1948</v>
+      </c>
+      <c r="E88" s="125" t="s">
         <v>1949</v>
       </c>
-      <c r="E88" s="125" t="s">
+      <c r="F88" s="17" t="s">
         <v>1950</v>
       </c>
-      <c r="F88" s="17" t="s">
+      <c r="G88" s="127" t="s">
+        <v>1805</v>
+      </c>
+      <c r="H88" s="125" t="s">
         <v>1951</v>
-      </c>
-      <c r="G88" s="127" t="s">
-        <v>1806</v>
-      </c>
-      <c r="H88" s="125" t="s">
-        <v>1952</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="15" t="s">
-        <v>1957</v>
+        <v>1956</v>
       </c>
       <c r="C89" s="15"/>
       <c r="D89" s="15"/>
       <c r="E89" s="125" t="s">
-        <v>1958</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B90" s="13" t="s">
-        <v>1959</v>
+        <v>1958</v>
       </c>
       <c r="C90" s="14"/>
       <c r="D90" s="14"/>
@@ -34919,30 +34917,30 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B91" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C91" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C91" s="16" t="s">
+      <c r="D91" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D91" s="16" t="s">
+      <c r="E91" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E91" s="16" t="s">
+      <c r="F91" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F91" s="16" t="s">
+      <c r="G91" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G91" s="16" t="s">
+      <c r="H91" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H91" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B92" s="25" t="s">
-        <v>1960</v>
+        <v>1959</v>
       </c>
       <c r="C92" s="128" t="n">
         <v>0.7</v>
@@ -34951,21 +34949,21 @@
         <v>75</v>
       </c>
       <c r="E92" s="125" t="s">
-        <v>1961</v>
+        <v>1960</v>
       </c>
       <c r="F92" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G92" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H92" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B93" s="25" t="s">
-        <v>1962</v>
+        <v>1961</v>
       </c>
       <c r="C93" s="128" t="n">
         <v>0.4</v>
@@ -34974,67 +34972,67 @@
         <v>75</v>
       </c>
       <c r="E93" s="125" t="s">
-        <v>1963</v>
+        <v>1962</v>
       </c>
       <c r="F93" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G93" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H93" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B94" s="25" t="s">
-        <v>1964</v>
+        <v>1963</v>
       </c>
       <c r="C94" s="132" t="n">
         <v>365</v>
       </c>
       <c r="D94" s="17" t="s">
+        <v>1964</v>
+      </c>
+      <c r="E94" s="125" t="s">
         <v>1965</v>
       </c>
-      <c r="E94" s="125" t="s">
-        <v>1966</v>
-      </c>
       <c r="F94" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G94" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H94" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B95" s="25" t="s">
-        <v>1967</v>
+        <v>1966</v>
       </c>
       <c r="C95" s="128" t="n">
         <v>0.8</v>
       </c>
       <c r="D95" s="17" t="s">
-        <v>1968</v>
+        <v>1967</v>
       </c>
       <c r="E95" s="125" t="s">
-        <v>1966</v>
+        <v>1965</v>
       </c>
       <c r="F95" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G95" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H95" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B96" s="13" t="s">
-        <v>1969</v>
+        <v>1968</v>
       </c>
       <c r="C96" s="14"/>
       <c r="D96" s="14"/>
@@ -35045,53 +35043,53 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B97" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C97" s="16" t="s">
         <v>1787</v>
       </c>
-      <c r="C97" s="16" t="s">
+      <c r="D97" s="16" t="s">
         <v>1788</v>
       </c>
-      <c r="D97" s="16" t="s">
+      <c r="E97" s="16" t="s">
         <v>1789</v>
       </c>
-      <c r="E97" s="16" t="s">
+      <c r="F97" s="16" t="s">
         <v>1790</v>
       </c>
-      <c r="F97" s="16" t="s">
+      <c r="G97" s="16" t="s">
         <v>1791</v>
       </c>
-      <c r="G97" s="16" t="s">
+      <c r="H97" s="16" t="s">
         <v>1792</v>
-      </c>
-      <c r="H97" s="16" t="s">
-        <v>1793</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B98" s="25" t="s">
-        <v>1970</v>
+        <v>1969</v>
       </c>
       <c r="C98" s="132" t="n">
         <v>1200</v>
       </c>
       <c r="D98" s="17" t="s">
+        <v>1970</v>
+      </c>
+      <c r="E98" s="125" t="s">
         <v>1971</v>
       </c>
-      <c r="E98" s="125" t="s">
-        <v>1972</v>
-      </c>
       <c r="F98" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G98" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H98" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B99" s="25" t="s">
-        <v>1973</v>
+        <v>1972</v>
       </c>
       <c r="C99" s="132" t="n">
         <v>60</v>
@@ -35100,21 +35098,21 @@
         <v>150</v>
       </c>
       <c r="E99" s="125" t="s">
-        <v>1972</v>
+        <v>1971</v>
       </c>
       <c r="F99" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G99" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H99" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B100" s="25" t="s">
-        <v>1974</v>
+        <v>1973</v>
       </c>
       <c r="C100" s="132" t="n">
         <v>5</v>
@@ -35123,21 +35121,21 @@
         <v>82</v>
       </c>
       <c r="E100" s="125" t="s">
-        <v>1972</v>
+        <v>1971</v>
       </c>
       <c r="F100" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G100" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H100" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B101" s="25" t="s">
-        <v>1975</v>
+        <v>1974</v>
       </c>
       <c r="C101" s="132" t="n">
         <v>10</v>
@@ -35146,21 +35144,21 @@
         <v>82</v>
       </c>
       <c r="E101" s="125" t="s">
-        <v>1972</v>
+        <v>1971</v>
       </c>
       <c r="F101" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G101" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H101" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B102" s="25" t="s">
-        <v>1976</v>
+        <v>1975</v>
       </c>
       <c r="C102" s="132" t="n">
         <v>15</v>
@@ -35169,21 +35167,21 @@
         <v>82</v>
       </c>
       <c r="E102" s="125" t="s">
-        <v>1972</v>
+        <v>1971</v>
       </c>
       <c r="F102" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G102" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H102" s="125" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B103" s="25" t="s">
-        <v>1977</v>
+        <v>1976</v>
       </c>
       <c r="C103" s="138" t="n">
         <v>1.645</v>
@@ -35192,30 +35190,30 @@
         <v>75</v>
       </c>
       <c r="E103" s="125" t="s">
-        <v>1978</v>
+        <v>1977</v>
       </c>
       <c r="F103" s="17" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G103" s="125" t="s">
         <v>3</v>
       </c>
       <c r="H103" s="125" t="s">
-        <v>1979</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B104" s="25" t="s">
+        <v>1979</v>
+      </c>
+      <c r="C104" s="133" t="s">
         <v>1980</v>
-      </c>
-      <c r="C104" s="133" t="s">
-        <v>1981</v>
       </c>
       <c r="D104" s="12" t="s">
         <v>75</v>
       </c>
       <c r="E104" s="134" t="s">
-        <v>1982</v>
+        <v>1981</v>
       </c>
       <c r="G104" s="52" t="s">
         <v>3</v>
@@ -35223,16 +35221,16 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B105" s="25" t="s">
+        <v>1982</v>
+      </c>
+      <c r="C105" s="133" t="s">
         <v>1983</v>
-      </c>
-      <c r="C105" s="133" t="s">
-        <v>1984</v>
       </c>
       <c r="D105" s="12" t="s">
         <v>75</v>
       </c>
       <c r="E105" s="134" t="s">
-        <v>1982</v>
+        <v>1981</v>
       </c>
       <c r="G105" s="52" t="s">
         <v>3</v>
@@ -35240,16 +35238,16 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B106" s="25" t="s">
+        <v>1984</v>
+      </c>
+      <c r="C106" s="133" t="s">
         <v>1985</v>
-      </c>
-      <c r="C106" s="133" t="s">
-        <v>1986</v>
       </c>
       <c r="D106" s="12" t="s">
         <v>75</v>
       </c>
       <c r="E106" s="134" t="s">
-        <v>1982</v>
+        <v>1981</v>
       </c>
       <c r="G106" s="52" t="s">
         <v>3</v>
@@ -35410,7 +35408,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B123" s="13" t="s">
-        <v>1987</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>